<commit_message>
Actualización automática de datos 2026-09-25 02:06
</commit_message>
<xml_diff>
--- a/datos_congreso.xlsx
+++ b/datos_congreso.xlsx
@@ -545,7 +545,7 @@
         </is>
       </c>
       <c r="B7" s="5" t="n">
-        <v>69</v>
+        <v>73</v>
       </c>
     </row>
     <row r="8">
@@ -556,7 +556,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-24</t>
         </is>
       </c>
     </row>
@@ -567,7 +567,7 @@
         </is>
       </c>
       <c r="B9" s="6" t="n">
-        <v>0.9379999999999999</v>
+        <v>0.9350000000000001</v>
       </c>
     </row>
     <row r="10">
@@ -577,7 +577,7 @@
         </is>
       </c>
       <c r="B10" s="6" t="n">
-        <v>0.985</v>
+        <v>0.982</v>
       </c>
     </row>
     <row r="11">
@@ -587,7 +587,7 @@
         </is>
       </c>
       <c r="B11" s="5" t="n">
-        <v>633</v>
+        <v>700</v>
       </c>
     </row>
     <row r="12">
@@ -597,7 +597,7 @@
         </is>
       </c>
       <c r="B12" s="5" t="n">
-        <v>142</v>
+        <v>178</v>
       </c>
     </row>
     <row r="13">
@@ -1098,7 +1098,7 @@
         </is>
       </c>
       <c r="D7" s="11" t="n">
-        <v>0.88</v>
+        <v>0.89</v>
       </c>
       <c r="E7" s="11" t="n">
         <v>1</v>
@@ -1221,13 +1221,13 @@
         </is>
       </c>
       <c r="D10" s="11" t="n">
-        <v>0.86</v>
+        <v>0.82</v>
       </c>
       <c r="E10" s="11" t="n">
         <v>1</v>
       </c>
       <c r="F10" s="10" t="n">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="G10" s="10" t="n">
         <v>0</v>
@@ -1303,16 +1303,16 @@
         </is>
       </c>
       <c r="D12" s="11" t="n">
-        <v>1</v>
+        <v>0.98</v>
       </c>
       <c r="E12" s="11" t="n">
-        <v>1</v>
+        <v>0.98</v>
       </c>
       <c r="F12" s="10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G12" s="10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H12" s="12" t="n">
         <v>14210997</v>
@@ -1344,7 +1344,7 @@
         </is>
       </c>
       <c r="D13" s="11" t="n">
-        <v>0.89</v>
+        <v>0.9</v>
       </c>
       <c r="E13" s="11" t="n">
         <v>1</v>
@@ -1385,13 +1385,13 @@
         </is>
       </c>
       <c r="D14" s="11" t="n">
-        <v>0.98</v>
+        <v>0.93</v>
       </c>
       <c r="E14" s="11" t="n">
         <v>1</v>
       </c>
       <c r="F14" s="10" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="G14" s="10" t="n">
         <v>0</v>
@@ -1716,13 +1716,13 @@
         <v>0.86</v>
       </c>
       <c r="E22" s="11" t="n">
-        <v>0.98</v>
+        <v>0.97</v>
       </c>
       <c r="F22" s="10" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="G22" s="10" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H22" s="12" t="n">
         <v>11878311</v>
@@ -1877,13 +1877,13 @@
         </is>
       </c>
       <c r="D26" s="11" t="n">
-        <v>0.47</v>
+        <v>0.45</v>
       </c>
       <c r="E26" s="11" t="n">
         <v>0.98</v>
       </c>
       <c r="F26" s="10" t="n">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="G26" s="10" t="n">
         <v>1</v>
@@ -2000,16 +2000,16 @@
         </is>
       </c>
       <c r="D29" s="11" t="n">
-        <v>0.92</v>
+        <v>0.91</v>
       </c>
       <c r="E29" s="11" t="n">
-        <v>0.95</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="F29" s="10" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G29" s="10" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H29" s="12" t="n">
         <v>16084693</v>
@@ -2246,7 +2246,7 @@
         </is>
       </c>
       <c r="D35" s="11" t="n">
-        <v>0.88</v>
+        <v>0.89</v>
       </c>
       <c r="E35" s="11" t="n">
         <v>0.95</v>
@@ -2328,16 +2328,16 @@
         </is>
       </c>
       <c r="D37" s="11" t="n">
+        <v>0.9399999999999999</v>
+      </c>
+      <c r="E37" s="11" t="n">
         <v>0.95</v>
       </c>
-      <c r="E37" s="11" t="n">
-        <v>0.97</v>
-      </c>
       <c r="F37" s="10" t="n">
+        <v>4</v>
+      </c>
+      <c r="G37" s="10" t="n">
         <v>3</v>
-      </c>
-      <c r="G37" s="10" t="n">
-        <v>2</v>
       </c>
       <c r="H37" s="12" t="n">
         <v>14264411</v>
@@ -2492,16 +2492,16 @@
         </is>
       </c>
       <c r="D41" s="11" t="n">
-        <v>0.95</v>
+        <v>0.9</v>
       </c>
       <c r="E41" s="11" t="n">
-        <v>1</v>
+        <v>0.98</v>
       </c>
       <c r="F41" s="10" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="G41" s="10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H41" s="12" t="n">
         <v>16748295</v>
@@ -3066,16 +3066,16 @@
         </is>
       </c>
       <c r="D55" s="11" t="n">
-        <v>0.97</v>
+        <v>0.91</v>
       </c>
       <c r="E55" s="11" t="n">
-        <v>1</v>
+        <v>0.98</v>
       </c>
       <c r="F55" s="10" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="G55" s="10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H55" s="12" t="n">
         <v>14240910</v>
@@ -3271,13 +3271,13 @@
         </is>
       </c>
       <c r="D60" s="11" t="n">
-        <v>0.98</v>
+        <v>0.95</v>
       </c>
       <c r="E60" s="11" t="n">
         <v>1</v>
       </c>
       <c r="F60" s="10" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G60" s="10" t="n">
         <v>0</v>
@@ -3394,16 +3394,16 @@
         </is>
       </c>
       <c r="D63" s="11" t="n">
-        <v>0.95</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="E63" s="11" t="n">
-        <v>0.95</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="F63" s="10" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G63" s="10" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H63" s="12" t="n">
         <v>13853861</v>
@@ -3435,16 +3435,16 @@
         </is>
       </c>
       <c r="D64" s="11" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.93</v>
       </c>
       <c r="E64" s="11" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.93</v>
       </c>
       <c r="F64" s="10" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G64" s="10" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H64" s="12" t="n">
         <v>12055366</v>
@@ -3517,10 +3517,10 @@
         </is>
       </c>
       <c r="D66" s="11" t="n">
-        <v>0.82</v>
+        <v>0.83</v>
       </c>
       <c r="E66" s="11" t="n">
-        <v>0.92</v>
+        <v>0.93</v>
       </c>
       <c r="F66" s="10" t="n">
         <v>12</v>
@@ -3599,16 +3599,16 @@
         </is>
       </c>
       <c r="D68" s="11" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.89</v>
       </c>
       <c r="E68" s="11" t="n">
-        <v>0.95</v>
+        <v>0.9</v>
       </c>
       <c r="F68" s="10" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="G68" s="10" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="H68" s="12" t="n">
         <v>8078582</v>
@@ -3763,10 +3763,10 @@
         </is>
       </c>
       <c r="D72" s="11" t="n">
-        <v>0.88</v>
+        <v>0.89</v>
       </c>
       <c r="E72" s="11" t="n">
-        <v>0.92</v>
+        <v>0.93</v>
       </c>
       <c r="F72" s="10" t="n">
         <v>8</v>
@@ -4009,7 +4009,7 @@
         </is>
       </c>
       <c r="D78" s="11" t="n">
-        <v>0.92</v>
+        <v>0.93</v>
       </c>
       <c r="E78" s="11" t="n">
         <v>0.9399999999999999</v>
@@ -4050,7 +4050,7 @@
         </is>
       </c>
       <c r="D79" s="11" t="n">
-        <v>0.92</v>
+        <v>0.93</v>
       </c>
       <c r="E79" s="11" t="n">
         <v>0.98</v>
@@ -4132,7 +4132,7 @@
         </is>
       </c>
       <c r="D81" s="11" t="n">
-        <v>0.88</v>
+        <v>0.89</v>
       </c>
       <c r="E81" s="11" t="n">
         <v>0.97</v>
@@ -4261,7 +4261,7 @@
         <v>1</v>
       </c>
       <c r="F84" s="10" t="n">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="G84" s="10" t="n">
         <v>0</v>
@@ -4337,7 +4337,7 @@
         </is>
       </c>
       <c r="D86" s="11" t="n">
-        <v>0.92</v>
+        <v>0.93</v>
       </c>
       <c r="E86" s="11" t="n">
         <v>0.9399999999999999</v>
@@ -4378,7 +4378,7 @@
         </is>
       </c>
       <c r="D87" s="11" t="n">
-        <v>0.92</v>
+        <v>0.93</v>
       </c>
       <c r="E87" s="11" t="n">
         <v>0.98</v>
@@ -4419,7 +4419,7 @@
         </is>
       </c>
       <c r="D88" s="11" t="n">
-        <v>0.76</v>
+        <v>0.78</v>
       </c>
       <c r="E88" s="11" t="n">
         <v>1</v>
@@ -4911,16 +4911,16 @@
         </is>
       </c>
       <c r="D100" s="11" t="n">
-        <v>0.52</v>
+        <v>0.49</v>
       </c>
       <c r="E100" s="11" t="n">
-        <v>1</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="F100" s="10" t="n">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="G100" s="10" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H100" s="12" t="n">
         <v>15301662</v>
@@ -4952,7 +4952,7 @@
         </is>
       </c>
       <c r="D101" s="11" t="n">
-        <v>0.92</v>
+        <v>0.93</v>
       </c>
       <c r="E101" s="11" t="n">
         <v>0.98</v>
@@ -5198,7 +5198,7 @@
         </is>
       </c>
       <c r="D107" s="11" t="n">
-        <v>0.92</v>
+        <v>0.93</v>
       </c>
       <c r="E107" s="11" t="n">
         <v>1</v>
@@ -5239,7 +5239,7 @@
         </is>
       </c>
       <c r="D108" s="11" t="n">
-        <v>0.89</v>
+        <v>0.9</v>
       </c>
       <c r="E108" s="11" t="n">
         <v>1</v>
@@ -5403,10 +5403,10 @@
         </is>
       </c>
       <c r="D112" s="11" t="n">
-        <v>0.88</v>
+        <v>0.89</v>
       </c>
       <c r="E112" s="11" t="n">
-        <v>0.92</v>
+        <v>0.93</v>
       </c>
       <c r="F112" s="10" t="n">
         <v>8</v>
@@ -5444,13 +5444,13 @@
         </is>
       </c>
       <c r="D113" s="11" t="n">
-        <v>0.85</v>
+        <v>0.83</v>
       </c>
       <c r="E113" s="11" t="n">
         <v>0.98</v>
       </c>
       <c r="F113" s="10" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="G113" s="10" t="n">
         <v>5</v>
@@ -5485,16 +5485,16 @@
         </is>
       </c>
       <c r="D114" s="11" t="n">
-        <v>0.76</v>
+        <v>0.72</v>
       </c>
       <c r="E114" s="11" t="n">
-        <v>0.98</v>
+        <v>0.93</v>
       </c>
       <c r="F114" s="10" t="n">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="G114" s="10" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="H114" s="12" t="n">
         <v>11262742</v>
@@ -5532,7 +5532,7 @@
         <v>1</v>
       </c>
       <c r="F115" s="10" t="n">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="G115" s="10" t="n">
         <v>0</v>
@@ -5608,10 +5608,10 @@
         </is>
       </c>
       <c r="D117" s="11" t="n">
-        <v>0.88</v>
+        <v>0.89</v>
       </c>
       <c r="E117" s="11" t="n">
-        <v>0.88</v>
+        <v>0.89</v>
       </c>
       <c r="F117" s="10" t="n">
         <v>8</v>
@@ -5693,13 +5693,13 @@
         <v>0.75</v>
       </c>
       <c r="E119" s="11" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.93</v>
       </c>
       <c r="F119" s="10" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="G119" s="10" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H119" s="12" t="n">
         <v>14935706</v>
@@ -5731,16 +5731,16 @@
         </is>
       </c>
       <c r="D120" s="11" t="n">
-        <v>0.97</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="E120" s="11" t="n">
-        <v>0.97</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="F120" s="10" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G120" s="10" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H120" s="12" t="n">
         <v>14830525</v>
@@ -5936,7 +5936,7 @@
         </is>
       </c>
       <c r="D125" s="11" t="n">
-        <v>0.8100000000000001</v>
+        <v>0.82</v>
       </c>
       <c r="E125" s="11" t="n">
         <v>0.9399999999999999</v>
@@ -6182,16 +6182,16 @@
         </is>
       </c>
       <c r="D131" s="11" t="n">
-        <v>1</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="E131" s="11" t="n">
-        <v>1</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="F131" s="10" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="G131" s="10" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H131" s="12" t="n">
         <v>12704015</v>
@@ -6346,7 +6346,7 @@
         </is>
       </c>
       <c r="D135" s="11" t="n">
-        <v>0.85</v>
+        <v>0.86</v>
       </c>
       <c r="E135" s="11" t="n">
         <v>1</v>
@@ -6674,16 +6674,16 @@
         </is>
       </c>
       <c r="D143" s="11" t="n">
-        <v>0.97</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="E143" s="11" t="n">
-        <v>1</v>
+        <v>0.98</v>
       </c>
       <c r="F143" s="10" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G143" s="10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H143" s="12" t="n">
         <v>13352251</v>
@@ -6715,16 +6715,16 @@
         </is>
       </c>
       <c r="D144" s="11" t="n">
-        <v>0.92</v>
+        <v>0.87</v>
       </c>
       <c r="E144" s="11" t="n">
-        <v>0.98</v>
+        <v>0.93</v>
       </c>
       <c r="F144" s="10" t="n">
+        <v>9</v>
+      </c>
+      <c r="G144" s="10" t="n">
         <v>5</v>
-      </c>
-      <c r="G144" s="10" t="n">
-        <v>1</v>
       </c>
       <c r="H144" s="12" t="n">
         <v>12416605</v>
@@ -6756,7 +6756,7 @@
         </is>
       </c>
       <c r="D145" s="11" t="n">
-        <v>0.92</v>
+        <v>0.93</v>
       </c>
       <c r="E145" s="11" t="n">
         <v>0.98</v>
@@ -6879,7 +6879,7 @@
         </is>
       </c>
       <c r="D148" s="11" t="n">
-        <v>0.92</v>
+        <v>0.93</v>
       </c>
       <c r="E148" s="11" t="n">
         <v>1</v>
@@ -7084,7 +7084,7 @@
         </is>
       </c>
       <c r="D153" s="11" t="n">
-        <v>0.88</v>
+        <v>0.89</v>
       </c>
       <c r="E153" s="11" t="n">
         <v>1</v>
@@ -7207,16 +7207,16 @@
         </is>
       </c>
       <c r="D156" s="11" t="n">
-        <v>1</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="E156" s="11" t="n">
-        <v>1</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="F156" s="10" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="G156" s="10" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H156" s="12" t="n">
         <v>15982197</v>
@@ -7302,13 +7302,13 @@
         <v>7</v>
       </c>
       <c r="C2" s="11" t="n">
-        <v>0.9790000000000001</v>
+        <v>0.97</v>
       </c>
       <c r="D2" s="12" t="n">
-        <v>1.4</v>
+        <v>2</v>
       </c>
       <c r="E2" s="12" t="n">
-        <v>0.3</v>
+        <v>0.9</v>
       </c>
       <c r="F2" s="12" t="n">
         <v>14893179</v>
@@ -7320,101 +7320,101 @@
     <row r="3">
       <c r="A3" s="10" t="inlineStr">
         <is>
-          <t>PPD</t>
+          <t>Republicanos</t>
         </is>
       </c>
       <c r="B3" s="10" t="n">
-        <v>4</v>
+        <v>28</v>
       </c>
       <c r="C3" s="11" t="n">
-        <v>0.972</v>
+        <v>0.965</v>
       </c>
       <c r="D3" s="12" t="n">
-        <v>1.8</v>
+        <v>2.3</v>
       </c>
       <c r="E3" s="12" t="n">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="F3" s="12" t="n">
-        <v>14929578</v>
+        <v>12895816</v>
       </c>
       <c r="G3" s="12" t="n">
-        <v>59718312</v>
+        <v>361082848</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="10" t="inlineStr">
         <is>
-          <t>Republicanos</t>
+          <t>UDI</t>
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>28</v>
+        <v>13</v>
       </c>
       <c r="C4" s="11" t="n">
-        <v>0.9690000000000001</v>
+        <v>0.9640000000000001</v>
       </c>
       <c r="D4" s="12" t="n">
-        <v>2</v>
+        <v>2.5</v>
       </c>
       <c r="E4" s="12" t="n">
-        <v>0.7</v>
+        <v>1</v>
       </c>
       <c r="F4" s="12" t="n">
-        <v>12895816</v>
+        <v>13348033</v>
       </c>
       <c r="G4" s="12" t="n">
-        <v>361082848</v>
+        <v>173524429</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="10" t="inlineStr">
         <is>
-          <t>UDI</t>
+          <t>PS/PL/PR</t>
         </is>
       </c>
       <c r="B5" s="10" t="n">
         <v>13</v>
       </c>
       <c r="C5" s="11" t="n">
-        <v>0.966</v>
+        <v>0.9590000000000001</v>
       </c>
       <c r="D5" s="12" t="n">
-        <v>2.2</v>
+        <v>2.7</v>
       </c>
       <c r="E5" s="12" t="n">
-        <v>0.7</v>
+        <v>0.8</v>
       </c>
       <c r="F5" s="12" t="n">
-        <v>13348033</v>
+        <v>15233287</v>
       </c>
       <c r="G5" s="12" t="n">
-        <v>173524429</v>
+        <v>198032731</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="10" t="inlineStr">
         <is>
-          <t>PS/PL/PR</t>
+          <t>PPD</t>
         </is>
       </c>
       <c r="B6" s="10" t="n">
-        <v>13</v>
+        <v>4</v>
       </c>
       <c r="C6" s="11" t="n">
-        <v>0.965</v>
+        <v>0.958</v>
       </c>
       <c r="D6" s="12" t="n">
-        <v>2.2</v>
+        <v>2.8</v>
       </c>
       <c r="E6" s="12" t="n">
-        <v>0.6</v>
+        <v>1.8</v>
       </c>
       <c r="F6" s="12" t="n">
-        <v>15233287</v>
+        <v>14929578</v>
       </c>
       <c r="G6" s="12" t="n">
-        <v>198032731</v>
+        <v>59718312</v>
       </c>
     </row>
     <row r="7">
@@ -7427,10 +7427,10 @@
         <v>13</v>
       </c>
       <c r="C7" s="11" t="n">
-        <v>0.9490000000000001</v>
+        <v>0.948</v>
       </c>
       <c r="D7" s="12" t="n">
-        <v>3.2</v>
+        <v>3.5</v>
       </c>
       <c r="E7" s="12" t="n">
         <v>1.2</v>
@@ -7445,126 +7445,126 @@
     <row r="8">
       <c r="A8" s="10" t="inlineStr">
         <is>
-          <t>Comunistas</t>
+          <t>PNL</t>
         </is>
       </c>
       <c r="B8" s="10" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C8" s="11" t="n">
-        <v>0.948</v>
+        <v>0.945</v>
       </c>
       <c r="D8" s="12" t="n">
-        <v>3.4</v>
+        <v>3.8</v>
       </c>
       <c r="E8" s="12" t="n">
-        <v>1</v>
+        <v>1.9</v>
       </c>
       <c r="F8" s="12" t="n">
-        <v>15236021</v>
+        <v>14164351</v>
       </c>
       <c r="G8" s="12" t="n">
-        <v>137124189</v>
+        <v>113314808</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="10" t="inlineStr">
         <is>
-          <t>PNL</t>
+          <t>Independientes</t>
         </is>
       </c>
       <c r="B9" s="10" t="n">
-        <v>8</v>
+        <v>29</v>
       </c>
       <c r="C9" s="11" t="n">
-        <v>0.945</v>
+        <v>0.9420000000000001</v>
       </c>
       <c r="D9" s="12" t="n">
-        <v>3.6</v>
+        <v>4.1</v>
       </c>
       <c r="E9" s="12" t="n">
-        <v>1.8</v>
+        <v>1</v>
       </c>
       <c r="F9" s="12" t="n">
-        <v>14164351</v>
+        <v>14636885</v>
       </c>
       <c r="G9" s="12" t="n">
-        <v>113314808</v>
+        <v>424469665</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="10" t="inlineStr">
         <is>
-          <t>Independientes</t>
+          <t>Comunistas</t>
         </is>
       </c>
       <c r="B10" s="10" t="n">
-        <v>29</v>
+        <v>9</v>
       </c>
       <c r="C10" s="11" t="n">
-        <v>0.9429999999999999</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="D10" s="12" t="n">
-        <v>3.9</v>
+        <v>4.2</v>
       </c>
       <c r="E10" s="12" t="n">
-        <v>0.9</v>
+        <v>1.2</v>
       </c>
       <c r="F10" s="12" t="n">
-        <v>14636885</v>
+        <v>15236021</v>
       </c>
       <c r="G10" s="12" t="n">
-        <v>424469665</v>
+        <v>137124189</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="10" t="inlineStr">
         <is>
-          <t>PDG</t>
+          <t>Demócratas/Amarillos</t>
         </is>
       </c>
       <c r="B11" s="10" t="n">
-        <v>14</v>
+        <v>1</v>
       </c>
       <c r="C11" s="11" t="n">
-        <v>0.929</v>
+        <v>0.93</v>
       </c>
       <c r="D11" s="12" t="n">
-        <v>4.7</v>
+        <v>5</v>
       </c>
       <c r="E11" s="12" t="n">
-        <v>0.9</v>
+        <v>4</v>
       </c>
       <c r="F11" s="12" t="n">
-        <v>14875781</v>
+        <v>15457599</v>
       </c>
       <c r="G11" s="12" t="n">
-        <v>208260934</v>
+        <v>15457599</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="10" t="inlineStr">
         <is>
-          <t>Demócratas/Amarillos</t>
+          <t>PDG</t>
         </is>
       </c>
       <c r="B12" s="10" t="n">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="C12" s="11" t="n">
-        <v>0.92</v>
+        <v>0.929</v>
       </c>
       <c r="D12" s="12" t="n">
         <v>5</v>
       </c>
       <c r="E12" s="12" t="n">
-        <v>4</v>
+        <v>1.1</v>
       </c>
       <c r="F12" s="12" t="n">
-        <v>15457599</v>
+        <v>14875781</v>
       </c>
       <c r="G12" s="12" t="n">
-        <v>15457599</v>
+        <v>208260934</v>
       </c>
     </row>
     <row r="13">
@@ -7577,13 +7577,13 @@
         <v>16</v>
       </c>
       <c r="C13" s="11" t="n">
-        <v>0.797</v>
+        <v>0.7959999999999999</v>
       </c>
       <c r="D13" s="12" t="n">
-        <v>13.7</v>
+        <v>14.6</v>
       </c>
       <c r="E13" s="12" t="n">
-        <v>1.2</v>
+        <v>1.4</v>
       </c>
       <c r="F13" s="12" t="n">
         <v>14792325</v>
@@ -9474,7 +9474,7 @@
         <v>1</v>
       </c>
       <c r="H7" s="11" t="n">
-        <v>0.88</v>
+        <v>0.89</v>
       </c>
       <c r="I7" s="11" t="n">
         <v>1</v>
@@ -9588,7 +9588,7 @@
         <v>1</v>
       </c>
       <c r="H10" s="11" t="n">
-        <v>0.86</v>
+        <v>0.82</v>
       </c>
       <c r="I10" s="11" t="n">
         <v>1</v>
@@ -9664,14 +9664,14 @@
         <v>1</v>
       </c>
       <c r="H12" s="11" t="n">
-        <v>1</v>
+        <v>0.98</v>
       </c>
       <c r="I12" s="11" t="n">
-        <v>1</v>
+        <v>0.98</v>
       </c>
       <c r="J12" s="10" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No (licencias/permisos)</t>
         </is>
       </c>
     </row>
@@ -9702,7 +9702,7 @@
         <v>1</v>
       </c>
       <c r="H13" s="11" t="n">
-        <v>0.89</v>
+        <v>0.9</v>
       </c>
       <c r="I13" s="11" t="n">
         <v>1</v>
@@ -9740,7 +9740,7 @@
         <v>1</v>
       </c>
       <c r="H14" s="11" t="n">
-        <v>0.98</v>
+        <v>0.93</v>
       </c>
       <c r="I14" s="11" t="n">
         <v>1</v>
@@ -10047,7 +10047,7 @@
         <v>0.86</v>
       </c>
       <c r="I22" s="11" t="n">
-        <v>0.98</v>
+        <v>0.97</v>
       </c>
       <c r="J22" s="10" t="inlineStr">
         <is>
@@ -10196,7 +10196,7 @@
         <v>0.985</v>
       </c>
       <c r="H26" s="11" t="n">
-        <v>0.47</v>
+        <v>0.45</v>
       </c>
       <c r="I26" s="11" t="n">
         <v>0.98</v>
@@ -10310,14 +10310,14 @@
         <v>0.955</v>
       </c>
       <c r="H29" s="11" t="n">
-        <v>0.92</v>
+        <v>0.91</v>
       </c>
       <c r="I29" s="11" t="n">
-        <v>0.95</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="J29" s="10" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No (licencias/permisos)</t>
         </is>
       </c>
     </row>
@@ -10538,7 +10538,7 @@
         <v>0.97</v>
       </c>
       <c r="H35" s="11" t="n">
-        <v>0.88</v>
+        <v>0.89</v>
       </c>
       <c r="I35" s="11" t="n">
         <v>0.95</v>
@@ -10614,14 +10614,14 @@
         <v>0.97</v>
       </c>
       <c r="H37" s="11" t="n">
+        <v>0.9399999999999999</v>
+      </c>
+      <c r="I37" s="11" t="n">
         <v>0.95</v>
       </c>
-      <c r="I37" s="11" t="n">
-        <v>0.97</v>
-      </c>
       <c r="J37" s="10" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No (licencias/permisos)</t>
         </is>
       </c>
     </row>
@@ -10766,14 +10766,14 @@
         <v>1</v>
       </c>
       <c r="H41" s="11" t="n">
-        <v>0.95</v>
+        <v>0.9</v>
       </c>
       <c r="I41" s="11" t="n">
-        <v>1</v>
+        <v>0.98</v>
       </c>
       <c r="J41" s="10" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No (licencias/permisos)</t>
         </is>
       </c>
     </row>
@@ -11298,14 +11298,14 @@
         <v>1</v>
       </c>
       <c r="H55" s="11" t="n">
-        <v>0.97</v>
+        <v>0.91</v>
       </c>
       <c r="I55" s="11" t="n">
-        <v>1</v>
+        <v>0.98</v>
       </c>
       <c r="J55" s="10" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No (licencias/permisos)</t>
         </is>
       </c>
     </row>
@@ -11488,7 +11488,7 @@
         <v>1</v>
       </c>
       <c r="H60" s="11" t="n">
-        <v>0.98</v>
+        <v>0.95</v>
       </c>
       <c r="I60" s="11" t="n">
         <v>1</v>
@@ -11602,14 +11602,14 @@
         <v>0.955</v>
       </c>
       <c r="H63" s="11" t="n">
-        <v>0.95</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="I63" s="11" t="n">
-        <v>0.95</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="J63" s="10" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No (licencias/permisos)</t>
         </is>
       </c>
     </row>
@@ -11640,14 +11640,14 @@
         <v>0.9259999999999999</v>
       </c>
       <c r="H64" s="11" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.93</v>
       </c>
       <c r="I64" s="11" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.93</v>
       </c>
       <c r="J64" s="10" t="inlineStr">
         <is>
-          <t>No (licencias/permisos)</t>
+          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -11716,10 +11716,10 @@
         <v>0.892</v>
       </c>
       <c r="H66" s="11" t="n">
-        <v>0.82</v>
+        <v>0.83</v>
       </c>
       <c r="I66" s="11" t="n">
-        <v>0.92</v>
+        <v>0.93</v>
       </c>
       <c r="J66" s="10" t="inlineStr">
         <is>
@@ -11792,14 +11792,14 @@
         <v>0.955</v>
       </c>
       <c r="H68" s="11" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.89</v>
       </c>
       <c r="I68" s="11" t="n">
-        <v>0.95</v>
+        <v>0.9</v>
       </c>
       <c r="J68" s="10" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No (licencias/permisos)</t>
         </is>
       </c>
     </row>
@@ -11944,10 +11944,10 @@
         <v>0.9279999999999999</v>
       </c>
       <c r="H72" s="11" t="n">
-        <v>0.88</v>
+        <v>0.89</v>
       </c>
       <c r="I72" s="11" t="n">
-        <v>0.92</v>
+        <v>0.93</v>
       </c>
       <c r="J72" s="10" t="inlineStr">
         <is>
@@ -12172,7 +12172,7 @@
         <v>0.9259999999999999</v>
       </c>
       <c r="H78" s="11" t="n">
-        <v>0.92</v>
+        <v>0.93</v>
       </c>
       <c r="I78" s="11" t="n">
         <v>0.9399999999999999</v>
@@ -12210,7 +12210,7 @@
         <v>0.985</v>
       </c>
       <c r="H79" s="11" t="n">
-        <v>0.92</v>
+        <v>0.93</v>
       </c>
       <c r="I79" s="11" t="n">
         <v>0.98</v>
@@ -12286,7 +12286,7 @@
         <v>0.97</v>
       </c>
       <c r="H81" s="11" t="n">
-        <v>0.88</v>
+        <v>0.89</v>
       </c>
       <c r="I81" s="11" t="n">
         <v>0.97</v>
@@ -12476,7 +12476,7 @@
         <v>0.9399999999999999</v>
       </c>
       <c r="H86" s="11" t="n">
-        <v>0.92</v>
+        <v>0.93</v>
       </c>
       <c r="I86" s="11" t="n">
         <v>0.9399999999999999</v>
@@ -12514,7 +12514,7 @@
         <v>0.986</v>
       </c>
       <c r="H87" s="11" t="n">
-        <v>0.92</v>
+        <v>0.93</v>
       </c>
       <c r="I87" s="11" t="n">
         <v>0.98</v>
@@ -12552,7 +12552,7 @@
         <v>1</v>
       </c>
       <c r="H88" s="11" t="n">
-        <v>0.76</v>
+        <v>0.78</v>
       </c>
       <c r="I88" s="11" t="n">
         <v>1</v>
@@ -13008,14 +13008,14 @@
         <v>1</v>
       </c>
       <c r="H100" s="11" t="n">
-        <v>0.52</v>
+        <v>0.49</v>
       </c>
       <c r="I100" s="11" t="n">
-        <v>1</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="J100" s="10" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No (licencias/permisos)</t>
         </is>
       </c>
     </row>
@@ -13046,7 +13046,7 @@
         <v>0.985</v>
       </c>
       <c r="H101" s="11" t="n">
-        <v>0.92</v>
+        <v>0.93</v>
       </c>
       <c r="I101" s="11" t="n">
         <v>0.98</v>
@@ -13274,7 +13274,7 @@
         <v>1</v>
       </c>
       <c r="H107" s="11" t="n">
-        <v>0.92</v>
+        <v>0.93</v>
       </c>
       <c r="I107" s="11" t="n">
         <v>1</v>
@@ -13312,7 +13312,7 @@
         <v>1</v>
       </c>
       <c r="H108" s="11" t="n">
-        <v>0.89</v>
+        <v>0.9</v>
       </c>
       <c r="I108" s="11" t="n">
         <v>1</v>
@@ -13464,10 +13464,10 @@
         <v>0.925</v>
       </c>
       <c r="H112" s="11" t="n">
-        <v>0.88</v>
+        <v>0.89</v>
       </c>
       <c r="I112" s="11" t="n">
-        <v>0.92</v>
+        <v>0.93</v>
       </c>
       <c r="J112" s="10" t="inlineStr">
         <is>
@@ -13502,7 +13502,7 @@
         <v>1</v>
       </c>
       <c r="H113" s="11" t="n">
-        <v>0.85</v>
+        <v>0.83</v>
       </c>
       <c r="I113" s="11" t="n">
         <v>0.98</v>
@@ -13540,14 +13540,14 @@
         <v>0.985</v>
       </c>
       <c r="H114" s="11" t="n">
-        <v>0.76</v>
+        <v>0.72</v>
       </c>
       <c r="I114" s="11" t="n">
-        <v>0.98</v>
+        <v>0.93</v>
       </c>
       <c r="J114" s="10" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No (licencias/permisos)</t>
         </is>
       </c>
     </row>
@@ -13654,10 +13654,10 @@
         <v>0.8809999999999999</v>
       </c>
       <c r="H117" s="11" t="n">
-        <v>0.88</v>
+        <v>0.89</v>
       </c>
       <c r="I117" s="11" t="n">
-        <v>0.88</v>
+        <v>0.89</v>
       </c>
       <c r="J117" s="10" t="inlineStr">
         <is>
@@ -13733,11 +13733,11 @@
         <v>0.75</v>
       </c>
       <c r="I119" s="11" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.93</v>
       </c>
       <c r="J119" s="10" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No (licencias/permisos)</t>
         </is>
       </c>
     </row>
@@ -13768,10 +13768,10 @@
         <v>0.915</v>
       </c>
       <c r="H120" s="11" t="n">
-        <v>0.97</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="I120" s="11" t="n">
-        <v>0.97</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="J120" s="10" t="inlineStr">
         <is>
@@ -13958,7 +13958,7 @@
         <v>0.9399999999999999</v>
       </c>
       <c r="H125" s="11" t="n">
-        <v>0.8100000000000001</v>
+        <v>0.82</v>
       </c>
       <c r="I125" s="11" t="n">
         <v>0.9399999999999999</v>
@@ -14186,14 +14186,14 @@
         <v>1</v>
       </c>
       <c r="H131" s="11" t="n">
-        <v>1</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="I131" s="11" t="n">
-        <v>1</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="J131" s="10" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No (licencias/permisos)</t>
         </is>
       </c>
     </row>
@@ -14338,7 +14338,7 @@
         <v>1</v>
       </c>
       <c r="H135" s="11" t="n">
-        <v>0.85</v>
+        <v>0.86</v>
       </c>
       <c r="I135" s="11" t="n">
         <v>1</v>
@@ -14642,14 +14642,14 @@
         <v>1</v>
       </c>
       <c r="H143" s="11" t="n">
-        <v>0.97</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="I143" s="11" t="n">
-        <v>1</v>
+        <v>0.98</v>
       </c>
       <c r="J143" s="10" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No (licencias/permisos)</t>
         </is>
       </c>
     </row>
@@ -14680,14 +14680,14 @@
         <v>0.985</v>
       </c>
       <c r="H144" s="11" t="n">
-        <v>0.92</v>
+        <v>0.87</v>
       </c>
       <c r="I144" s="11" t="n">
-        <v>0.98</v>
+        <v>0.93</v>
       </c>
       <c r="J144" s="10" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No (licencias/permisos)</t>
         </is>
       </c>
     </row>
@@ -14718,7 +14718,7 @@
         <v>0.985</v>
       </c>
       <c r="H145" s="11" t="n">
-        <v>0.92</v>
+        <v>0.93</v>
       </c>
       <c r="I145" s="11" t="n">
         <v>0.98</v>
@@ -14832,7 +14832,7 @@
         <v>1</v>
       </c>
       <c r="H148" s="11" t="n">
-        <v>0.92</v>
+        <v>0.93</v>
       </c>
       <c r="I148" s="11" t="n">
         <v>1</v>
@@ -15022,7 +15022,7 @@
         <v>1</v>
       </c>
       <c r="H153" s="11" t="n">
-        <v>0.88</v>
+        <v>0.89</v>
       </c>
       <c r="I153" s="11" t="n">
         <v>1</v>
@@ -15136,21 +15136,21 @@
         <v>1</v>
       </c>
       <c r="H156" s="11" t="n">
-        <v>1</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="I156" s="11" t="n">
-        <v>1</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="J156" s="10" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No (licencias/permisos)</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" s="15" t="inlineStr">
         <is>
-          <t>Conclusión: 143 de 155 diputad@s coinciden con el dato oficial en menos de 1 punto porcentual.</t>
+          <t>Conclusión: 130 de 155 diputad@s coinciden con el dato oficial en menos de 1 punto porcentual.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualización automática de datos 2026-10-16 01:37
</commit_message>
<xml_diff>
--- a/datos_congreso.xlsx
+++ b/datos_congreso.xlsx
@@ -1,19 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumen" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Diputados" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bancadas" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Votaciones 2026" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Destacadas" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Senado-Presidencia" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Asistencia oficial camara.cl" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Resumen" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Diputados" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Bancadas" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Votaciones 2026" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Destacadas" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Senado-Presidencia" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Asistencia oficial camara.cl" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Diputados'!$A$1:$K$156</definedName>
@@ -545,7 +545,7 @@
         </is>
       </c>
       <c r="B7" s="5" t="n">
-        <v>73</v>
+        <v>80</v>
       </c>
     </row>
     <row r="8">
@@ -556,7 +556,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-10-15</t>
         </is>
       </c>
     </row>
@@ -567,7 +567,7 @@
         </is>
       </c>
       <c r="B9" s="6" t="n">
-        <v>0.9350000000000001</v>
+        <v>0.9329999999999999</v>
       </c>
     </row>
     <row r="10">
@@ -577,7 +577,7 @@
         </is>
       </c>
       <c r="B10" s="6" t="n">
-        <v>0.982</v>
+        <v>0.983</v>
       </c>
     </row>
     <row r="11">
@@ -587,7 +587,7 @@
         </is>
       </c>
       <c r="B11" s="5" t="n">
-        <v>700</v>
+        <v>801</v>
       </c>
     </row>
     <row r="12">
@@ -597,7 +597,7 @@
         </is>
       </c>
       <c r="B12" s="5" t="n">
-        <v>178</v>
+        <v>185</v>
       </c>
     </row>
     <row r="13">
@@ -655,7 +655,7 @@
         </is>
       </c>
       <c r="B19" s="5" t="n">
-        <v>976</v>
+        <v>1028</v>
       </c>
     </row>
     <row r="20">
@@ -665,7 +665,7 @@
         </is>
       </c>
       <c r="B20" s="5" t="n">
-        <v>777</v>
+        <v>814</v>
       </c>
     </row>
     <row r="21">
@@ -675,7 +675,7 @@
         </is>
       </c>
       <c r="B21" s="5" t="n">
-        <v>199</v>
+        <v>214</v>
       </c>
     </row>
     <row r="22">
@@ -685,7 +685,7 @@
         </is>
       </c>
       <c r="B22" s="5" t="n">
-        <v>618</v>
+        <v>632</v>
       </c>
     </row>
     <row r="23">
@@ -879,7 +879,7 @@
     <row r="2">
       <c r="A2" s="10" t="inlineStr">
         <is>
-          <t>Agustín Romero</t>
+          <t>Agustín Romero Leiva</t>
         </is>
       </c>
       <c r="B2" s="10" t="inlineStr">
@@ -893,13 +893,13 @@
         </is>
       </c>
       <c r="D2" s="11" t="n">
-        <v>0.97</v>
+        <v>0.92</v>
       </c>
       <c r="E2" s="11" t="n">
         <v>0.97</v>
       </c>
       <c r="F2" s="10" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="G2" s="10" t="n">
         <v>2</v>
@@ -920,7 +920,7 @@
     <row r="3">
       <c r="A3" s="10" t="inlineStr">
         <is>
-          <t>Alejandra Valdebenito</t>
+          <t>Alejandra Valdebenito Torres</t>
         </is>
       </c>
       <c r="B3" s="10" t="inlineStr">
@@ -961,7 +961,7 @@
     <row r="4">
       <c r="A4" s="10" t="inlineStr">
         <is>
-          <t>Alejandro Bernales</t>
+          <t>Alejandro Bernales Maldonado</t>
         </is>
       </c>
       <c r="B4" s="10" t="inlineStr">
@@ -1002,7 +1002,7 @@
     <row r="5">
       <c r="A5" s="10" t="inlineStr">
         <is>
-          <t>Alejandro Riquelme</t>
+          <t>Alejandro Riquelme Ducci</t>
         </is>
       </c>
       <c r="B5" s="10" t="inlineStr">
@@ -1043,7 +1043,7 @@
     <row r="6">
       <c r="A6" s="10" t="inlineStr">
         <is>
-          <t>Alex Nahuelquin</t>
+          <t>Alex Nahuelquin Nahuelquin</t>
         </is>
       </c>
       <c r="B6" s="10" t="inlineStr">
@@ -1084,7 +1084,7 @@
     <row r="7">
       <c r="A7" s="10" t="inlineStr">
         <is>
-          <t>Ana María Gazmuri</t>
+          <t>Ana María Gazmuri Vieira</t>
         </is>
       </c>
       <c r="B7" s="10" t="inlineStr">
@@ -1098,13 +1098,13 @@
         </is>
       </c>
       <c r="D7" s="11" t="n">
-        <v>0.89</v>
+        <v>0.86</v>
       </c>
       <c r="E7" s="11" t="n">
         <v>1</v>
       </c>
       <c r="F7" s="10" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="G7" s="10" t="n">
         <v>0</v>
@@ -1125,7 +1125,7 @@
     <row r="8">
       <c r="A8" s="10" t="inlineStr">
         <is>
-          <t>Andrea Macías</t>
+          <t>Andrea Macías Palma</t>
         </is>
       </c>
       <c r="B8" s="10" t="inlineStr">
@@ -1166,7 +1166,7 @@
     <row r="9">
       <c r="A9" s="10" t="inlineStr">
         <is>
-          <t>Andrea Parra</t>
+          <t>Andrea Parra Sauterel</t>
         </is>
       </c>
       <c r="B9" s="10" t="inlineStr">
@@ -1207,7 +1207,7 @@
     <row r="10">
       <c r="A10" s="10" t="inlineStr">
         <is>
-          <t>Andrés Celis</t>
+          <t>Andrés Celis Montt</t>
         </is>
       </c>
       <c r="B10" s="10" t="inlineStr">
@@ -1221,16 +1221,16 @@
         </is>
       </c>
       <c r="D10" s="11" t="n">
-        <v>0.82</v>
+        <v>0.75</v>
       </c>
       <c r="E10" s="11" t="n">
-        <v>1</v>
+        <v>0.95</v>
       </c>
       <c r="F10" s="10" t="n">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="G10" s="10" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H10" s="12" t="n">
         <v>15103271</v>
@@ -1248,7 +1248,7 @@
     <row r="11">
       <c r="A11" s="10" t="inlineStr">
         <is>
-          <t>Benjamín Lorca</t>
+          <t>Benjamín Lorca Inzunza</t>
         </is>
       </c>
       <c r="B11" s="10" t="inlineStr">
@@ -1262,13 +1262,13 @@
         </is>
       </c>
       <c r="D11" s="11" t="n">
-        <v>1</v>
+        <v>0.97</v>
       </c>
       <c r="E11" s="11" t="n">
         <v>1</v>
       </c>
       <c r="F11" s="10" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G11" s="10" t="n">
         <v>0</v>
@@ -1289,7 +1289,7 @@
     <row r="12">
       <c r="A12" s="10" t="inlineStr">
         <is>
-          <t>Benjamín Moreno</t>
+          <t>Benjamín Moreno Bascur</t>
         </is>
       </c>
       <c r="B12" s="10" t="inlineStr">
@@ -1303,16 +1303,16 @@
         </is>
       </c>
       <c r="D12" s="11" t="n">
-        <v>0.98</v>
+        <v>0.96</v>
       </c>
       <c r="E12" s="11" t="n">
-        <v>0.98</v>
+        <v>0.97</v>
       </c>
       <c r="F12" s="10" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G12" s="10" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H12" s="12" t="n">
         <v>14210997</v>
@@ -1330,7 +1330,7 @@
     <row r="13">
       <c r="A13" s="10" t="inlineStr">
         <is>
-          <t>Bernardo Salinas</t>
+          <t>Bernardo Salinas Maya</t>
         </is>
       </c>
       <c r="B13" s="10" t="inlineStr">
@@ -1344,7 +1344,7 @@
         </is>
       </c>
       <c r="D13" s="11" t="n">
-        <v>0.9</v>
+        <v>0.91</v>
       </c>
       <c r="E13" s="11" t="n">
         <v>1</v>
@@ -1371,7 +1371,7 @@
     <row r="14">
       <c r="A14" s="10" t="inlineStr">
         <is>
-          <t>Boris Barrera</t>
+          <t>Boris Barrera Moreno</t>
         </is>
       </c>
       <c r="B14" s="10" t="inlineStr">
@@ -1385,13 +1385,13 @@
         </is>
       </c>
       <c r="D14" s="11" t="n">
-        <v>0.93</v>
+        <v>0.85</v>
       </c>
       <c r="E14" s="11" t="n">
         <v>1</v>
       </c>
       <c r="F14" s="10" t="n">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="G14" s="10" t="n">
         <v>0</v>
@@ -1412,7 +1412,7 @@
     <row r="15">
       <c r="A15" s="10" t="inlineStr">
         <is>
-          <t>Carlo Arqueros</t>
+          <t>Carlo Arqueros Pizarro</t>
         </is>
       </c>
       <c r="B15" s="10" t="inlineStr">
@@ -1453,7 +1453,7 @@
     <row r="16">
       <c r="A16" s="10" t="inlineStr">
         <is>
-          <t>Carlos Bianchi</t>
+          <t>Carlos Bianchi Chelech</t>
         </is>
       </c>
       <c r="B16" s="10" t="inlineStr">
@@ -1494,7 +1494,7 @@
     <row r="17">
       <c r="A17" s="10" t="inlineStr">
         <is>
-          <t>Carlos Carvajal</t>
+          <t>Carlos Carvajal Gallardo</t>
         </is>
       </c>
       <c r="B17" s="10" t="inlineStr">
@@ -1535,7 +1535,7 @@
     <row r="18">
       <c r="A18" s="10" t="inlineStr">
         <is>
-          <t>Carlos Chandía</t>
+          <t>Carlos Chandía Alarcón</t>
         </is>
       </c>
       <c r="B18" s="10" t="inlineStr">
@@ -1576,7 +1576,7 @@
     <row r="19">
       <c r="A19" s="10" t="inlineStr">
         <is>
-          <t>Carlos Cuadrado</t>
+          <t>Carlos Cuadrado Prats</t>
         </is>
       </c>
       <c r="B19" s="10" t="inlineStr">
@@ -1590,10 +1590,10 @@
         </is>
       </c>
       <c r="D19" s="11" t="n">
-        <v>0.95</v>
+        <v>0.96</v>
       </c>
       <c r="E19" s="11" t="n">
-        <v>0.95</v>
+        <v>0.96</v>
       </c>
       <c r="F19" s="10" t="n">
         <v>3</v>
@@ -1617,7 +1617,7 @@
     <row r="20">
       <c r="A20" s="10" t="inlineStr">
         <is>
-          <t>Carolina Cucumides</t>
+          <t>Carolina Cucumides Calderón</t>
         </is>
       </c>
       <c r="B20" s="10" t="inlineStr">
@@ -1658,7 +1658,7 @@
     <row r="21">
       <c r="A21" s="10" t="inlineStr">
         <is>
-          <t>Carolina Tello</t>
+          <t>Carolina Tello Rojas</t>
         </is>
       </c>
       <c r="B21" s="10" t="inlineStr">
@@ -1699,7 +1699,7 @@
     <row r="22">
       <c r="A22" s="10" t="inlineStr">
         <is>
-          <t>Catalina Del Real</t>
+          <t>Catalina Del Real Mihovilovic</t>
         </is>
       </c>
       <c r="B22" s="10" t="inlineStr">
@@ -1713,7 +1713,7 @@
         </is>
       </c>
       <c r="D22" s="11" t="n">
-        <v>0.86</v>
+        <v>0.87</v>
       </c>
       <c r="E22" s="11" t="n">
         <v>0.97</v>
@@ -1740,7 +1740,7 @@
     <row r="23">
       <c r="A23" s="10" t="inlineStr">
         <is>
-          <t>Chiara Barchiesi</t>
+          <t>Chiara Barchiesi Chávez</t>
         </is>
       </c>
       <c r="B23" s="10" t="inlineStr">
@@ -1754,10 +1754,10 @@
         </is>
       </c>
       <c r="D23" s="11" t="n">
-        <v>0.95</v>
+        <v>0.96</v>
       </c>
       <c r="E23" s="11" t="n">
-        <v>0.95</v>
+        <v>0.96</v>
       </c>
       <c r="F23" s="10" t="n">
         <v>3</v>
@@ -1781,7 +1781,7 @@
     <row r="24">
       <c r="A24" s="10" t="inlineStr">
         <is>
-          <t>Claudia Mora</t>
+          <t>Claudia Mora Vega</t>
         </is>
       </c>
       <c r="B24" s="10" t="inlineStr">
@@ -1822,7 +1822,7 @@
     <row r="25">
       <c r="A25" s="10" t="inlineStr">
         <is>
-          <t>Claudia Reyes</t>
+          <t>Claudia Reyes Larenas</t>
         </is>
       </c>
       <c r="B25" s="10" t="inlineStr">
@@ -1836,7 +1836,7 @@
         </is>
       </c>
       <c r="D25" s="11" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.95</v>
       </c>
       <c r="E25" s="11" t="n">
         <v>1</v>
@@ -1863,7 +1863,7 @@
     <row r="26">
       <c r="A26" s="10" t="inlineStr">
         <is>
-          <t>Coca Ericka Ñanco</t>
+          <t>Coca Ericka Ñanco Vásquez</t>
         </is>
       </c>
       <c r="B26" s="10" t="inlineStr">
@@ -1877,13 +1877,13 @@
         </is>
       </c>
       <c r="D26" s="11" t="n">
-        <v>0.45</v>
+        <v>0.41</v>
       </c>
       <c r="E26" s="11" t="n">
         <v>0.98</v>
       </c>
       <c r="F26" s="10" t="n">
-        <v>40</v>
+        <v>47</v>
       </c>
       <c r="G26" s="10" t="n">
         <v>1</v>
@@ -1904,7 +1904,7 @@
     <row r="27">
       <c r="A27" s="10" t="inlineStr">
         <is>
-          <t>Constanza Hube</t>
+          <t>Constanza Hube Portus</t>
         </is>
       </c>
       <c r="B27" s="10" t="inlineStr">
@@ -1945,7 +1945,7 @@
     <row r="28">
       <c r="A28" s="10" t="inlineStr">
         <is>
-          <t>Constanza Schonhaut</t>
+          <t>Constanza Schonhaut Soto</t>
         </is>
       </c>
       <c r="B28" s="10" t="inlineStr">
@@ -1959,7 +1959,7 @@
         </is>
       </c>
       <c r="D28" s="11" t="n">
-        <v>0.95</v>
+        <v>0.96</v>
       </c>
       <c r="E28" s="11" t="n">
         <v>1</v>
@@ -1986,7 +1986,7 @@
     <row r="29">
       <c r="A29" s="10" t="inlineStr">
         <is>
-          <t>Consuelo Veloso</t>
+          <t>Consuelo Veloso Ávila</t>
         </is>
       </c>
       <c r="B29" s="10" t="inlineStr">
@@ -2000,10 +2000,10 @@
         </is>
       </c>
       <c r="D29" s="11" t="n">
-        <v>0.91</v>
+        <v>0.92</v>
       </c>
       <c r="E29" s="11" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.95</v>
       </c>
       <c r="F29" s="10" t="n">
         <v>6</v>
@@ -2027,7 +2027,7 @@
     <row r="30">
       <c r="A30" s="10" t="inlineStr">
         <is>
-          <t>Cristian Contreras</t>
+          <t>Cristian Contreras Radovic</t>
         </is>
       </c>
       <c r="B30" s="10" t="inlineStr">
@@ -2068,7 +2068,7 @@
     <row r="31">
       <c r="A31" s="10" t="inlineStr">
         <is>
-          <t>Cristian Mella</t>
+          <t>Cristian Mella Andaur</t>
         </is>
       </c>
       <c r="B31" s="10" t="inlineStr">
@@ -2109,7 +2109,7 @@
     <row r="32">
       <c r="A32" s="10" t="inlineStr">
         <is>
-          <t>Cristian Menchaca</t>
+          <t>Cristian Menchaca Pinochet</t>
         </is>
       </c>
       <c r="B32" s="10" t="inlineStr">
@@ -2123,7 +2123,7 @@
         </is>
       </c>
       <c r="D32" s="11" t="n">
-        <v>0.95</v>
+        <v>0.96</v>
       </c>
       <c r="E32" s="11" t="n">
         <v>1</v>
@@ -2150,7 +2150,7 @@
     <row r="33">
       <c r="A33" s="10" t="inlineStr">
         <is>
-          <t>Cristian Neira</t>
+          <t>Cristian Neira Martínez</t>
         </is>
       </c>
       <c r="B33" s="10" t="inlineStr">
@@ -2191,7 +2191,7 @@
     <row r="34">
       <c r="A34" s="10" t="inlineStr">
         <is>
-          <t>Cristián Araya</t>
+          <t>Cristián Araya Lerdo de Tejada</t>
         </is>
       </c>
       <c r="B34" s="10" t="inlineStr">
@@ -2205,10 +2205,10 @@
         </is>
       </c>
       <c r="D34" s="11" t="n">
-        <v>0.91</v>
+        <v>0.92</v>
       </c>
       <c r="E34" s="11" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.95</v>
       </c>
       <c r="F34" s="10" t="n">
         <v>6</v>
@@ -2232,7 +2232,7 @@
     <row r="35">
       <c r="A35" s="10" t="inlineStr">
         <is>
-          <t>Cristián Tapia</t>
+          <t>Cristián Tapia Ramos</t>
         </is>
       </c>
       <c r="B35" s="10" t="inlineStr">
@@ -2246,13 +2246,13 @@
         </is>
       </c>
       <c r="D35" s="11" t="n">
-        <v>0.89</v>
+        <v>0.88</v>
       </c>
       <c r="E35" s="11" t="n">
-        <v>0.95</v>
+        <v>0.96</v>
       </c>
       <c r="F35" s="10" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G35" s="10" t="n">
         <v>3</v>
@@ -2273,7 +2273,7 @@
     <row r="36">
       <c r="A36" s="10" t="inlineStr">
         <is>
-          <t>Cristóbal Martínez</t>
+          <t>Cristóbal Martínez Ramírez</t>
         </is>
       </c>
       <c r="B36" s="10" t="inlineStr">
@@ -2287,13 +2287,13 @@
         </is>
       </c>
       <c r="D36" s="11" t="n">
-        <v>0.95</v>
+        <v>0.91</v>
       </c>
       <c r="E36" s="11" t="n">
         <v>1</v>
       </c>
       <c r="F36" s="10" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="G36" s="10" t="n">
         <v>0</v>
@@ -2314,7 +2314,7 @@
     <row r="37">
       <c r="A37" s="10" t="inlineStr">
         <is>
-          <t>Cristóbal Urruticoechea</t>
+          <t>Cristóbal Urruticoechea Ríos</t>
         </is>
       </c>
       <c r="B37" s="10" t="inlineStr">
@@ -2328,10 +2328,10 @@
         </is>
       </c>
       <c r="D37" s="11" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.95</v>
       </c>
       <c r="E37" s="11" t="n">
-        <v>0.95</v>
+        <v>0.96</v>
       </c>
       <c r="F37" s="10" t="n">
         <v>4</v>
@@ -2355,7 +2355,7 @@
     <row r="38">
       <c r="A38" s="10" t="inlineStr">
         <is>
-          <t>César Valenzuela</t>
+          <t>César Valenzuela Maass</t>
         </is>
       </c>
       <c r="B38" s="10" t="inlineStr">
@@ -2396,7 +2396,7 @@
     <row r="39">
       <c r="A39" s="10" t="inlineStr">
         <is>
-          <t>Daniel Bustos</t>
+          <t>Daniel Bustos Leal</t>
         </is>
       </c>
       <c r="B39" s="10" t="inlineStr">
@@ -2437,7 +2437,7 @@
     <row r="40">
       <c r="A40" s="10" t="inlineStr">
         <is>
-          <t>Daniel Lilayu</t>
+          <t>Daniel Lilayu Vivanco</t>
         </is>
       </c>
       <c r="B40" s="10" t="inlineStr">
@@ -2478,7 +2478,7 @@
     <row r="41">
       <c r="A41" s="10" t="inlineStr">
         <is>
-          <t>Daniel Manouchehri</t>
+          <t>Daniel Manouchehri Lobos</t>
         </is>
       </c>
       <c r="B41" s="10" t="inlineStr">
@@ -2495,13 +2495,13 @@
         <v>0.9</v>
       </c>
       <c r="E41" s="11" t="n">
-        <v>0.98</v>
+        <v>1</v>
       </c>
       <c r="F41" s="10" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G41" s="10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H41" s="12" t="n">
         <v>16748295</v>
@@ -2519,7 +2519,7 @@
     <row r="42">
       <c r="A42" s="10" t="inlineStr">
         <is>
-          <t>Daniel Valenzuela</t>
+          <t>Daniel Valenzuela Salazar</t>
         </is>
       </c>
       <c r="B42" s="10" t="inlineStr">
@@ -2533,10 +2533,10 @@
         </is>
       </c>
       <c r="D42" s="11" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.95</v>
       </c>
       <c r="E42" s="11" t="n">
-        <v>0.95</v>
+        <v>0.96</v>
       </c>
       <c r="F42" s="10" t="n">
         <v>4</v>
@@ -2560,7 +2560,7 @@
     <row r="43">
       <c r="A43" s="10" t="inlineStr">
         <is>
-          <t>Daniela Serrano</t>
+          <t>Daniela Serrano Salazar</t>
         </is>
       </c>
       <c r="B43" s="10" t="inlineStr">
@@ -2601,7 +2601,7 @@
     <row r="44">
       <c r="A44" s="10" t="inlineStr">
         <is>
-          <t>Diego Schalper</t>
+          <t>Diego Schalper Sepúlveda</t>
         </is>
       </c>
       <c r="B44" s="10" t="inlineStr">
@@ -2615,10 +2615,10 @@
         </is>
       </c>
       <c r="D44" s="11" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.95</v>
       </c>
       <c r="E44" s="11" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.95</v>
       </c>
       <c r="F44" s="10" t="n">
         <v>4</v>
@@ -2642,7 +2642,7 @@
     <row r="45">
       <c r="A45" s="10" t="inlineStr">
         <is>
-          <t>Diego Vergara</t>
+          <t>Diego Vergara Rodríguez</t>
         </is>
       </c>
       <c r="B45" s="10" t="inlineStr">
@@ -2683,7 +2683,7 @@
     <row r="46">
       <c r="A46" s="10" t="inlineStr">
         <is>
-          <t>Eduardo Cretton</t>
+          <t>Eduardo Cretton Rebolledo</t>
         </is>
       </c>
       <c r="B46" s="10" t="inlineStr">
@@ -2724,7 +2724,7 @@
     <row r="47">
       <c r="A47" s="10" t="inlineStr">
         <is>
-          <t>Eduardo Durán</t>
+          <t>Eduardo Durán Salinas</t>
         </is>
       </c>
       <c r="B47" s="10" t="inlineStr">
@@ -2765,7 +2765,7 @@
     <row r="48">
       <c r="A48" s="10" t="inlineStr">
         <is>
-          <t>Eileen Urqueta</t>
+          <t>Eileen Urqueta Rojas</t>
         </is>
       </c>
       <c r="B48" s="10" t="inlineStr">
@@ -2806,7 +2806,7 @@
     <row r="49">
       <c r="A49" s="10" t="inlineStr">
         <is>
-          <t>Emilia Nuyado</t>
+          <t>Emilia Nuyado Ancapichun</t>
         </is>
       </c>
       <c r="B49" s="10" t="inlineStr">
@@ -2847,7 +2847,7 @@
     <row r="50">
       <c r="A50" s="10" t="inlineStr">
         <is>
-          <t>Emilia Schneider</t>
+          <t>Emilia Schneider Videla</t>
         </is>
       </c>
       <c r="B50" s="10" t="inlineStr">
@@ -2888,7 +2888,7 @@
     <row r="51">
       <c r="A51" s="10" t="inlineStr">
         <is>
-          <t>Enrique Bassaletti</t>
+          <t>Enrique Bassaletti Riess</t>
         </is>
       </c>
       <c r="B51" s="10" t="inlineStr">
@@ -2929,7 +2929,7 @@
     <row r="52">
       <c r="A52" s="10" t="inlineStr">
         <is>
-          <t>Erich Grohs</t>
+          <t>Erich Grohs Marín</t>
         </is>
       </c>
       <c r="B52" s="10" t="inlineStr">
@@ -2943,16 +2943,16 @@
         </is>
       </c>
       <c r="D52" s="11" t="n">
-        <v>0.91</v>
+        <v>0.88</v>
       </c>
       <c r="E52" s="11" t="n">
-        <v>0.95</v>
+        <v>0.93</v>
       </c>
       <c r="F52" s="10" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="G52" s="10" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H52" s="12" t="n">
         <v>14064893</v>
@@ -2970,7 +2970,7 @@
     <row r="53">
       <c r="A53" s="10" t="inlineStr">
         <is>
-          <t>Fabián Ossandón</t>
+          <t>Fabián Ossandón Briceño</t>
         </is>
       </c>
       <c r="B53" s="10" t="inlineStr">
@@ -2984,10 +2984,10 @@
         </is>
       </c>
       <c r="D53" s="11" t="n">
-        <v>0.95</v>
+        <v>0.96</v>
       </c>
       <c r="E53" s="11" t="n">
-        <v>0.95</v>
+        <v>0.96</v>
       </c>
       <c r="F53" s="10" t="n">
         <v>3</v>
@@ -3011,7 +3011,7 @@
     <row r="54">
       <c r="A54" s="10" t="inlineStr">
         <is>
-          <t>Felipe Camaño</t>
+          <t>Felipe Camaño Cárdenas</t>
         </is>
       </c>
       <c r="B54" s="10" t="inlineStr">
@@ -3025,7 +3025,7 @@
         </is>
       </c>
       <c r="D54" s="11" t="n">
-        <v>0.91</v>
+        <v>0.92</v>
       </c>
       <c r="E54" s="11" t="n">
         <v>1</v>
@@ -3052,7 +3052,7 @@
     <row r="55">
       <c r="A55" s="10" t="inlineStr">
         <is>
-          <t>Felipe Ross</t>
+          <t>Felipe Ross Correa</t>
         </is>
       </c>
       <c r="B55" s="10" t="inlineStr">
@@ -3072,7 +3072,7 @@
         <v>0.98</v>
       </c>
       <c r="F55" s="10" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G55" s="10" t="n">
         <v>1</v>
@@ -3093,7 +3093,7 @@
     <row r="56">
       <c r="A56" s="10" t="inlineStr">
         <is>
-          <t>Fernando Ugarte</t>
+          <t>Fernando Ugarte Tejeda</t>
         </is>
       </c>
       <c r="B56" s="10" t="inlineStr">
@@ -3134,7 +3134,7 @@
     <row r="57">
       <c r="A57" s="10" t="inlineStr">
         <is>
-          <t>Fernando Zamorano</t>
+          <t>Fernando Zamorano Peralta</t>
         </is>
       </c>
       <c r="B57" s="10" t="inlineStr">
@@ -3148,7 +3148,7 @@
         </is>
       </c>
       <c r="D57" s="11" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.95</v>
       </c>
       <c r="E57" s="11" t="n">
         <v>1</v>
@@ -3175,7 +3175,7 @@
     <row r="58">
       <c r="A58" s="10" t="inlineStr">
         <is>
-          <t>Flor Contreras</t>
+          <t>Flor Contreras Vivallo</t>
         </is>
       </c>
       <c r="B58" s="10" t="inlineStr">
@@ -3216,7 +3216,7 @@
     <row r="59">
       <c r="A59" s="10" t="inlineStr">
         <is>
-          <t>Flor Weisse</t>
+          <t>Flor Weisse Novoa</t>
         </is>
       </c>
       <c r="B59" s="10" t="inlineStr">
@@ -3230,13 +3230,13 @@
         </is>
       </c>
       <c r="D59" s="11" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.9</v>
       </c>
       <c r="E59" s="11" t="n">
         <v>1</v>
       </c>
       <c r="F59" s="10" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="G59" s="10" t="n">
         <v>0</v>
@@ -3257,7 +3257,7 @@
     <row r="60">
       <c r="A60" s="10" t="inlineStr">
         <is>
-          <t>Francesca Muñoz</t>
+          <t>Francesca Muñoz González</t>
         </is>
       </c>
       <c r="B60" s="10" t="inlineStr">
@@ -3271,7 +3271,7 @@
         </is>
       </c>
       <c r="D60" s="11" t="n">
-        <v>0.95</v>
+        <v>0.97</v>
       </c>
       <c r="E60" s="11" t="n">
         <v>1</v>
@@ -3298,7 +3298,7 @@
     <row r="61">
       <c r="A61" s="10" t="inlineStr">
         <is>
-          <t>Francisco Crisóstomo</t>
+          <t>Francisco Crisóstomo Llanos</t>
         </is>
       </c>
       <c r="B61" s="10" t="inlineStr">
@@ -3339,7 +3339,7 @@
     <row r="62">
       <c r="A62" s="10" t="inlineStr">
         <is>
-          <t>Francisco Orrego</t>
+          <t>Francisco Orrego Gutiérrez</t>
         </is>
       </c>
       <c r="B62" s="10" t="inlineStr">
@@ -3380,7 +3380,7 @@
     <row r="63">
       <c r="A63" s="10" t="inlineStr">
         <is>
-          <t>Félix Bugueño</t>
+          <t>Félix Bugueño Sotelo</t>
         </is>
       </c>
       <c r="B63" s="10" t="inlineStr">
@@ -3394,10 +3394,10 @@
         </is>
       </c>
       <c r="D63" s="11" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.95</v>
       </c>
       <c r="E63" s="11" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.95</v>
       </c>
       <c r="F63" s="10" t="n">
         <v>4</v>
@@ -3421,7 +3421,7 @@
     <row r="64">
       <c r="A64" s="10" t="inlineStr">
         <is>
-          <t>Gael Yeomans</t>
+          <t>Gael Yeomans Araya</t>
         </is>
       </c>
       <c r="B64" s="10" t="inlineStr">
@@ -3462,7 +3462,7 @@
     <row r="65">
       <c r="A65" s="10" t="inlineStr">
         <is>
-          <t>Germán Verdugo</t>
+          <t>Germán Verdugo Soto</t>
         </is>
       </c>
       <c r="B65" s="10" t="inlineStr">
@@ -3503,7 +3503,7 @@
     <row r="66">
       <c r="A66" s="10" t="inlineStr">
         <is>
-          <t>Gloria Naveillan</t>
+          <t>Gloria Naveillan Arriagada</t>
         </is>
       </c>
       <c r="B66" s="10" t="inlineStr">
@@ -3517,16 +3517,16 @@
         </is>
       </c>
       <c r="D66" s="11" t="n">
-        <v>0.83</v>
+        <v>0.78</v>
       </c>
       <c r="E66" s="11" t="n">
-        <v>0.93</v>
+        <v>0.92</v>
       </c>
       <c r="F66" s="10" t="n">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="G66" s="10" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H66" s="12" t="n">
         <v>14776706</v>
@@ -3544,7 +3544,7 @@
     <row r="67">
       <c r="A67" s="10" t="inlineStr">
         <is>
-          <t>Gonzalo Winter</t>
+          <t>Gonzalo Winter Etcheberry</t>
         </is>
       </c>
       <c r="B67" s="10" t="inlineStr">
@@ -3558,7 +3558,7 @@
         </is>
       </c>
       <c r="D67" s="11" t="n">
-        <v>0.91</v>
+        <v>0.92</v>
       </c>
       <c r="E67" s="11" t="n">
         <v>0.98</v>
@@ -3585,7 +3585,7 @@
     <row r="68">
       <c r="A68" s="10" t="inlineStr">
         <is>
-          <t>Guillermo Ramírez</t>
+          <t>Guillermo Ramírez Diez</t>
         </is>
       </c>
       <c r="B68" s="10" t="inlineStr">
@@ -3599,16 +3599,16 @@
         </is>
       </c>
       <c r="D68" s="11" t="n">
-        <v>0.89</v>
+        <v>0.9</v>
       </c>
       <c r="E68" s="11" t="n">
-        <v>0.9</v>
+        <v>0.96</v>
       </c>
       <c r="F68" s="10" t="n">
         <v>8</v>
       </c>
       <c r="G68" s="10" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="H68" s="12" t="n">
         <v>8078582</v>
@@ -3626,7 +3626,7 @@
     <row r="69">
       <c r="A69" s="10" t="inlineStr">
         <is>
-          <t>Guillermo Valdés</t>
+          <t>Guillermo Valdés Carmona</t>
         </is>
       </c>
       <c r="B69" s="10" t="inlineStr">
@@ -3667,7 +3667,7 @@
     <row r="70">
       <c r="A70" s="10" t="inlineStr">
         <is>
-          <t>Gustavo Gatica</t>
+          <t>Gustavo Gatica Villarroel</t>
         </is>
       </c>
       <c r="B70" s="10" t="inlineStr">
@@ -3708,7 +3708,7 @@
     <row r="71">
       <c r="A71" s="10" t="inlineStr">
         <is>
-          <t>Hans Marowski</t>
+          <t>Hans Marowski Cuevas</t>
         </is>
       </c>
       <c r="B71" s="10" t="inlineStr">
@@ -3749,7 +3749,7 @@
     <row r="72">
       <c r="A72" s="10" t="inlineStr">
         <is>
-          <t>Hotuiti Teao</t>
+          <t>Hotuiti Teao Drago</t>
         </is>
       </c>
       <c r="B72" s="10" t="inlineStr">
@@ -3763,16 +3763,16 @@
         </is>
       </c>
       <c r="D72" s="11" t="n">
-        <v>0.89</v>
+        <v>0.88</v>
       </c>
       <c r="E72" s="11" t="n">
-        <v>0.93</v>
+        <v>0.92</v>
       </c>
       <c r="F72" s="10" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G72" s="10" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H72" s="12" t="n">
         <v>8911557</v>
@@ -3790,7 +3790,7 @@
     <row r="73">
       <c r="A73" s="10" t="inlineStr">
         <is>
-          <t>Héctor Barría</t>
+          <t>Héctor Barría Angulo</t>
         </is>
       </c>
       <c r="B73" s="10" t="inlineStr">
@@ -3804,7 +3804,7 @@
         </is>
       </c>
       <c r="D73" s="11" t="n">
-        <v>0.91</v>
+        <v>0.92</v>
       </c>
       <c r="E73" s="11" t="n">
         <v>0.98</v>
@@ -3831,7 +3831,7 @@
     <row r="74">
       <c r="A74" s="10" t="inlineStr">
         <is>
-          <t>Héctor Ulloa</t>
+          <t>Héctor Ulloa Aguilera</t>
         </is>
       </c>
       <c r="B74" s="10" t="inlineStr">
@@ -3845,7 +3845,7 @@
         </is>
       </c>
       <c r="D74" s="11" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.95</v>
       </c>
       <c r="E74" s="11" t="n">
         <v>1</v>
@@ -3872,7 +3872,7 @@
     <row r="75">
       <c r="A75" s="10" t="inlineStr">
         <is>
-          <t>Ignacio Achurra</t>
+          <t>Ignacio Achurra Díaz</t>
         </is>
       </c>
       <c r="B75" s="10" t="inlineStr">
@@ -3913,7 +3913,7 @@
     <row r="76">
       <c r="A76" s="10" t="inlineStr">
         <is>
-          <t>Ignacio Urcullú</t>
+          <t>Ignacio Urcullú Clèment-Lund</t>
         </is>
       </c>
       <c r="B76" s="10" t="inlineStr">
@@ -3927,13 +3927,13 @@
         </is>
       </c>
       <c r="D76" s="11" t="n">
-        <v>1</v>
+        <v>0.95</v>
       </c>
       <c r="E76" s="11" t="n">
         <v>1</v>
       </c>
       <c r="F76" s="10" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="G76" s="10" t="n">
         <v>0</v>
@@ -3954,7 +3954,7 @@
     <row r="77">
       <c r="A77" s="10" t="inlineStr">
         <is>
-          <t>Irací Hassler</t>
+          <t>Irací Hassler Jacob</t>
         </is>
       </c>
       <c r="B77" s="10" t="inlineStr">
@@ -3995,7 +3995,7 @@
     <row r="78">
       <c r="A78" s="10" t="inlineStr">
         <is>
-          <t>Jaime Araya</t>
+          <t>Jaime Araya Guerrero</t>
         </is>
       </c>
       <c r="B78" s="10" t="inlineStr">
@@ -4012,7 +4012,7 @@
         <v>0.93</v>
       </c>
       <c r="E78" s="11" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.95</v>
       </c>
       <c r="F78" s="10" t="n">
         <v>5</v>
@@ -4036,7 +4036,7 @@
     <row r="79">
       <c r="A79" s="10" t="inlineStr">
         <is>
-          <t>Jaime Bassa</t>
+          <t>Jaime Bassa Mercado</t>
         </is>
       </c>
       <c r="B79" s="10" t="inlineStr">
@@ -4077,7 +4077,7 @@
     <row r="80">
       <c r="A80" s="10" t="inlineStr">
         <is>
-          <t>Jaime Coloma</t>
+          <t>Jaime Coloma Álamos</t>
         </is>
       </c>
       <c r="B80" s="10" t="inlineStr">
@@ -4118,7 +4118,7 @@
     <row r="81">
       <c r="A81" s="10" t="inlineStr">
         <is>
-          <t>Jaime Mulet</t>
+          <t>Jaime Mulet Martínez</t>
         </is>
       </c>
       <c r="B81" s="10" t="inlineStr">
@@ -4132,7 +4132,7 @@
         </is>
       </c>
       <c r="D81" s="11" t="n">
-        <v>0.89</v>
+        <v>0.9</v>
       </c>
       <c r="E81" s="11" t="n">
         <v>0.97</v>
@@ -4159,7 +4159,7 @@
     <row r="82">
       <c r="A82" s="10" t="inlineStr">
         <is>
-          <t>Javier Muñoz</t>
+          <t>Javier Muñoz Riquelme</t>
         </is>
       </c>
       <c r="B82" s="10" t="inlineStr">
@@ -4200,7 +4200,7 @@
     <row r="83">
       <c r="A83" s="10" t="inlineStr">
         <is>
-          <t>Javier Olivares</t>
+          <t>Javier Olivares Avendaño</t>
         </is>
       </c>
       <c r="B83" s="10" t="inlineStr">
@@ -4241,7 +4241,7 @@
     <row r="84">
       <c r="A84" s="10" t="inlineStr">
         <is>
-          <t>Javiera Morales</t>
+          <t>Javiera Morales Alvarado</t>
         </is>
       </c>
       <c r="B84" s="10" t="inlineStr">
@@ -4255,13 +4255,13 @@
         </is>
       </c>
       <c r="D84" s="11" t="n">
-        <v>0.08</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="E84" s="11" t="n">
         <v>1</v>
       </c>
       <c r="F84" s="10" t="n">
-        <v>67</v>
+        <v>74</v>
       </c>
       <c r="G84" s="10" t="n">
         <v>0</v>
@@ -4282,7 +4282,7 @@
     <row r="85">
       <c r="A85" s="10" t="inlineStr">
         <is>
-          <t>Javiera Rodríguez</t>
+          <t>Javiera Rodríguez Pascual</t>
         </is>
       </c>
       <c r="B85" s="10" t="inlineStr">
@@ -4323,7 +4323,7 @@
     <row r="86">
       <c r="A86" s="10" t="inlineStr">
         <is>
-          <t>Joanna Pérez</t>
+          <t>Joanna Pérez Olea</t>
         </is>
       </c>
       <c r="B86" s="10" t="inlineStr">
@@ -4340,7 +4340,7 @@
         <v>0.93</v>
       </c>
       <c r="E86" s="11" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.95</v>
       </c>
       <c r="F86" s="10" t="n">
         <v>5</v>
@@ -4364,7 +4364,7 @@
     <row r="87">
       <c r="A87" s="10" t="inlineStr">
         <is>
-          <t>Jorge Alessandri</t>
+          <t>Jorge Alessandri Vergara</t>
         </is>
       </c>
       <c r="B87" s="10" t="inlineStr">
@@ -4378,16 +4378,16 @@
         </is>
       </c>
       <c r="D87" s="11" t="n">
-        <v>0.93</v>
+        <v>0.91</v>
       </c>
       <c r="E87" s="11" t="n">
-        <v>0.98</v>
+        <v>0.97</v>
       </c>
       <c r="F87" s="10" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="G87" s="10" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H87" s="12" t="n">
         <v>14918019</v>
@@ -4405,7 +4405,7 @@
     <row r="88">
       <c r="A88" s="10" t="inlineStr">
         <is>
-          <t>Jorge Brito</t>
+          <t>Jorge Brito Hasbún</t>
         </is>
       </c>
       <c r="B88" s="10" t="inlineStr">
@@ -4419,13 +4419,13 @@
         </is>
       </c>
       <c r="D88" s="11" t="n">
-        <v>0.78</v>
+        <v>0.75</v>
       </c>
       <c r="E88" s="11" t="n">
         <v>1</v>
       </c>
       <c r="F88" s="10" t="n">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="G88" s="10" t="n">
         <v>0</v>
@@ -4446,7 +4446,7 @@
     <row r="89">
       <c r="A89" s="10" t="inlineStr">
         <is>
-          <t>Jorge Díaz</t>
+          <t>Jorge Díaz Ibarra</t>
         </is>
       </c>
       <c r="B89" s="10" t="inlineStr">
@@ -4487,7 +4487,7 @@
     <row r="90">
       <c r="A90" s="10" t="inlineStr">
         <is>
-          <t>Jorge Guzmán</t>
+          <t>Jorge Guzmán Zepeda</t>
         </is>
       </c>
       <c r="B90" s="10" t="inlineStr">
@@ -4528,7 +4528,7 @@
     <row r="91">
       <c r="A91" s="10" t="inlineStr">
         <is>
-          <t>José Antonio Kast</t>
+          <t>José Antonio Kast Adriasola</t>
         </is>
       </c>
       <c r="B91" s="10" t="inlineStr">
@@ -4569,7 +4569,7 @@
     <row r="92">
       <c r="A92" s="10" t="inlineStr">
         <is>
-          <t>José Antonio Rivas</t>
+          <t>José Antonio Rivas Villalobos</t>
         </is>
       </c>
       <c r="B92" s="10" t="inlineStr">
@@ -4610,7 +4610,7 @@
     <row r="93">
       <c r="A93" s="10" t="inlineStr">
         <is>
-          <t>José Carlos Meza</t>
+          <t>José Carlos Meza Pereira</t>
         </is>
       </c>
       <c r="B93" s="10" t="inlineStr">
@@ -4624,7 +4624,7 @@
         </is>
       </c>
       <c r="D93" s="11" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.95</v>
       </c>
       <c r="E93" s="11" t="n">
         <v>1</v>
@@ -4651,7 +4651,7 @@
     <row r="94">
       <c r="A94" s="10" t="inlineStr">
         <is>
-          <t>José Montalva</t>
+          <t>José Montalva Feuerhake</t>
         </is>
       </c>
       <c r="B94" s="10" t="inlineStr">
@@ -4665,7 +4665,7 @@
         </is>
       </c>
       <c r="D94" s="11" t="n">
-        <v>0.95</v>
+        <v>0.96</v>
       </c>
       <c r="E94" s="11" t="n">
         <v>1</v>
@@ -4692,7 +4692,7 @@
     <row r="95">
       <c r="A95" s="10" t="inlineStr">
         <is>
-          <t>Juan Carlos Beltrán</t>
+          <t>Juan Carlos Beltrán Silva</t>
         </is>
       </c>
       <c r="B95" s="10" t="inlineStr">
@@ -4709,13 +4709,13 @@
         <v>0.91</v>
       </c>
       <c r="E95" s="11" t="n">
-        <v>1</v>
+        <v>0.98</v>
       </c>
       <c r="F95" s="10" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G95" s="10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H95" s="12" t="n">
         <v>15730769</v>
@@ -4733,7 +4733,7 @@
     <row r="96">
       <c r="A96" s="10" t="inlineStr">
         <is>
-          <t>Juan Irarrázaval</t>
+          <t>Juan Irarrázaval Rossel</t>
         </is>
       </c>
       <c r="B96" s="10" t="inlineStr">
@@ -4774,7 +4774,7 @@
     <row r="97">
       <c r="A97" s="10" t="inlineStr">
         <is>
-          <t>Juan Marcelo Valenzuela</t>
+          <t>Juan Marcelo Valenzuela Henríquez</t>
         </is>
       </c>
       <c r="B97" s="10" t="inlineStr">
@@ -4788,16 +4788,16 @@
         </is>
       </c>
       <c r="D97" s="11" t="n">
-        <v>0.97</v>
+        <v>0.96</v>
       </c>
       <c r="E97" s="11" t="n">
-        <v>0.97</v>
+        <v>0.96</v>
       </c>
       <c r="F97" s="10" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G97" s="10" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H97" s="12" t="n">
         <v>14160335</v>
@@ -4815,7 +4815,7 @@
     <row r="98">
       <c r="A98" s="10" t="inlineStr">
         <is>
-          <t>Juan Santana</t>
+          <t>Juan Santana Castillo</t>
         </is>
       </c>
       <c r="B98" s="10" t="inlineStr">
@@ -4829,10 +4829,10 @@
         </is>
       </c>
       <c r="D98" s="11" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.95</v>
       </c>
       <c r="E98" s="11" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.95</v>
       </c>
       <c r="F98" s="10" t="n">
         <v>4</v>
@@ -4856,7 +4856,7 @@
     <row r="99">
       <c r="A99" s="10" t="inlineStr">
         <is>
-          <t>Leandro Kunstmann</t>
+          <t>Leandro Kunstmann Collado</t>
         </is>
       </c>
       <c r="B99" s="10" t="inlineStr">
@@ -4897,7 +4897,7 @@
     <row r="100">
       <c r="A100" s="10" t="inlineStr">
         <is>
-          <t>Lilian Betancurt</t>
+          <t>Lilian Betancurt Delgado</t>
         </is>
       </c>
       <c r="B100" s="10" t="inlineStr">
@@ -4911,16 +4911,16 @@
         </is>
       </c>
       <c r="D100" s="11" t="n">
-        <v>0.49</v>
+        <v>0.5</v>
       </c>
       <c r="E100" s="11" t="n">
-        <v>0.9399999999999999</v>
+        <v>1</v>
       </c>
       <c r="F100" s="10" t="n">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="G100" s="10" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="H100" s="12" t="n">
         <v>15301662</v>
@@ -4938,7 +4938,7 @@
     <row r="101">
       <c r="A101" s="10" t="inlineStr">
         <is>
-          <t>Lorena Fries</t>
+          <t>Lorena Fries Monleón</t>
         </is>
       </c>
       <c r="B101" s="10" t="inlineStr">
@@ -4979,7 +4979,7 @@
     <row r="102">
       <c r="A102" s="10" t="inlineStr">
         <is>
-          <t>Lorena Pizarro</t>
+          <t>Lorena Pizarro Sierra</t>
         </is>
       </c>
       <c r="B102" s="10" t="inlineStr">
@@ -5020,7 +5020,7 @@
     <row r="103">
       <c r="A103" s="10" t="inlineStr">
         <is>
-          <t>Luis Alberto Cuello</t>
+          <t>Luis Alberto Cuello Peña y Lillo</t>
         </is>
       </c>
       <c r="B103" s="10" t="inlineStr">
@@ -5061,7 +5061,7 @@
     <row r="104">
       <c r="A104" s="10" t="inlineStr">
         <is>
-          <t>Luis Malla</t>
+          <t>Luis Malla Valenzuela</t>
         </is>
       </c>
       <c r="B104" s="10" t="inlineStr">
@@ -5102,7 +5102,7 @@
     <row r="105">
       <c r="A105" s="10" t="inlineStr">
         <is>
-          <t>Luis Pardo</t>
+          <t>Luis Pardo Sáinz</t>
         </is>
       </c>
       <c r="B105" s="10" t="inlineStr">
@@ -5116,16 +5116,16 @@
         </is>
       </c>
       <c r="D105" s="11" t="n">
+        <v>0.97</v>
+      </c>
+      <c r="E105" s="11" t="n">
         <v>0.98</v>
       </c>
-      <c r="E105" s="11" t="n">
-        <v>1</v>
-      </c>
       <c r="F105" s="10" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G105" s="10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H105" s="12" t="n">
         <v>14991604</v>
@@ -5143,7 +5143,7 @@
     <row r="106">
       <c r="A106" s="10" t="inlineStr">
         <is>
-          <t>Luis Sánchez</t>
+          <t>Luis Sánchez Ossa</t>
         </is>
       </c>
       <c r="B106" s="10" t="inlineStr">
@@ -5184,7 +5184,7 @@
     <row r="107">
       <c r="A107" s="10" t="inlineStr">
         <is>
-          <t>Macarena Santelices</t>
+          <t>Macarena Santelices Cañas</t>
         </is>
       </c>
       <c r="B107" s="10" t="inlineStr">
@@ -5225,7 +5225,7 @@
     <row r="108">
       <c r="A108" s="10" t="inlineStr">
         <is>
-          <t>Marcela Hernando</t>
+          <t>Marcela Hernando Pérez</t>
         </is>
       </c>
       <c r="B108" s="10" t="inlineStr">
@@ -5239,7 +5239,7 @@
         </is>
       </c>
       <c r="D108" s="11" t="n">
-        <v>0.9</v>
+        <v>0.91</v>
       </c>
       <c r="E108" s="11" t="n">
         <v>1</v>
@@ -5266,7 +5266,7 @@
     <row r="109">
       <c r="A109" s="10" t="inlineStr">
         <is>
-          <t>Marco Antonio Sulantay</t>
+          <t>Marco Antonio Sulantay Olivares</t>
         </is>
       </c>
       <c r="B109" s="10" t="inlineStr">
@@ -5307,7 +5307,7 @@
     <row r="110">
       <c r="A110" s="10" t="inlineStr">
         <is>
-          <t>Marcos Barraza</t>
+          <t>Marcos Barraza Gómez</t>
         </is>
       </c>
       <c r="B110" s="10" t="inlineStr">
@@ -5348,7 +5348,7 @@
     <row r="111">
       <c r="A111" s="10" t="inlineStr">
         <is>
-          <t>Marcos Ilabaca</t>
+          <t>Marcos Ilabaca Cerda</t>
         </is>
       </c>
       <c r="B111" s="10" t="inlineStr">
@@ -5362,7 +5362,7 @@
         </is>
       </c>
       <c r="D111" s="11" t="n">
-        <v>0.91</v>
+        <v>0.92</v>
       </c>
       <c r="E111" s="11" t="n">
         <v>1</v>
@@ -5389,7 +5389,7 @@
     <row r="112">
       <c r="A112" s="10" t="inlineStr">
         <is>
-          <t>Mario Olavarría</t>
+          <t>Mario Olavarría Rodríguez</t>
         </is>
       </c>
       <c r="B112" s="10" t="inlineStr">
@@ -5403,7 +5403,7 @@
         </is>
       </c>
       <c r="D112" s="11" t="n">
-        <v>0.89</v>
+        <v>0.9</v>
       </c>
       <c r="E112" s="11" t="n">
         <v>0.93</v>
@@ -5430,7 +5430,7 @@
     <row r="113">
       <c r="A113" s="10" t="inlineStr">
         <is>
-          <t>Marisela Santibáñez</t>
+          <t>Marisela Santibáñez Novoa</t>
         </is>
       </c>
       <c r="B113" s="10" t="inlineStr">
@@ -5444,7 +5444,7 @@
         </is>
       </c>
       <c r="D113" s="11" t="n">
-        <v>0.83</v>
+        <v>0.86</v>
       </c>
       <c r="E113" s="11" t="n">
         <v>0.98</v>
@@ -5471,7 +5471,7 @@
     <row r="114">
       <c r="A114" s="10" t="inlineStr">
         <is>
-          <t>Marlene Pérez</t>
+          <t>Marlene Pérez Cartes</t>
         </is>
       </c>
       <c r="B114" s="10" t="inlineStr">
@@ -5485,16 +5485,16 @@
         </is>
       </c>
       <c r="D114" s="11" t="n">
-        <v>0.72</v>
+        <v>0.71</v>
       </c>
       <c r="E114" s="11" t="n">
-        <v>0.93</v>
+        <v>0.9</v>
       </c>
       <c r="F114" s="10" t="n">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="G114" s="10" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="H114" s="12" t="n">
         <v>11262742</v>
@@ -5512,7 +5512,7 @@
     <row r="115">
       <c r="A115" s="10" t="inlineStr">
         <is>
-          <t>María Francisca Bello</t>
+          <t>María Francisca Bello Campos</t>
         </is>
       </c>
       <c r="B115" s="10" t="inlineStr">
@@ -5532,7 +5532,7 @@
         <v>1</v>
       </c>
       <c r="F115" s="10" t="n">
-        <v>71</v>
+        <v>78</v>
       </c>
       <c r="G115" s="10" t="n">
         <v>0</v>
@@ -5553,7 +5553,7 @@
     <row r="116">
       <c r="A116" s="10" t="inlineStr">
         <is>
-          <t>Matías Fernández</t>
+          <t>Matías Fernández Hartwig</t>
         </is>
       </c>
       <c r="B116" s="10" t="inlineStr">
@@ -5594,7 +5594,7 @@
     <row r="117">
       <c r="A117" s="10" t="inlineStr">
         <is>
-          <t>Mauro González</t>
+          <t>Mauro González Villarroel</t>
         </is>
       </c>
       <c r="B117" s="10" t="inlineStr">
@@ -5608,10 +5608,10 @@
         </is>
       </c>
       <c r="D117" s="11" t="n">
-        <v>0.89</v>
+        <v>0.9</v>
       </c>
       <c r="E117" s="11" t="n">
-        <v>0.89</v>
+        <v>0.9</v>
       </c>
       <c r="F117" s="10" t="n">
         <v>8</v>
@@ -5635,7 +5635,7 @@
     <row r="118">
       <c r="A118" s="10" t="inlineStr">
         <is>
-          <t>Natalia Romero</t>
+          <t>Natalia Romero Talguia</t>
         </is>
       </c>
       <c r="B118" s="10" t="inlineStr">
@@ -5676,7 +5676,7 @@
     <row r="119">
       <c r="A119" s="10" t="inlineStr">
         <is>
-          <t>Nathalie Castillo</t>
+          <t>Nathalie Castillo Rojas</t>
         </is>
       </c>
       <c r="B119" s="10" t="inlineStr">
@@ -5690,16 +5690,16 @@
         </is>
       </c>
       <c r="D119" s="11" t="n">
-        <v>0.75</v>
+        <v>0.76</v>
       </c>
       <c r="E119" s="11" t="n">
-        <v>0.93</v>
+        <v>0.92</v>
       </c>
       <c r="F119" s="10" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="G119" s="10" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H119" s="12" t="n">
         <v>14935706</v>
@@ -5717,7 +5717,7 @@
     <row r="120">
       <c r="A120" s="10" t="inlineStr">
         <is>
-          <t>Nelson Venegas</t>
+          <t>Nelson Venegas Salazar</t>
         </is>
       </c>
       <c r="B120" s="10" t="inlineStr">
@@ -5731,10 +5731,10 @@
         </is>
       </c>
       <c r="D120" s="11" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.95</v>
       </c>
       <c r="E120" s="11" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.95</v>
       </c>
       <c r="F120" s="10" t="n">
         <v>4</v>
@@ -5758,7 +5758,7 @@
     <row r="121">
       <c r="A121" s="10" t="inlineStr">
         <is>
-          <t>Omar Sabat</t>
+          <t>Omar Sabat Guzmán</t>
         </is>
       </c>
       <c r="B121" s="10" t="inlineStr">
@@ -5799,7 +5799,7 @@
     <row r="122">
       <c r="A122" s="10" t="inlineStr">
         <is>
-          <t>Pamela Jiles</t>
+          <t>Pamela Jiles Moreno</t>
         </is>
       </c>
       <c r="B122" s="10" t="inlineStr">
@@ -5840,7 +5840,7 @@
     <row r="123">
       <c r="A123" s="10" t="inlineStr">
         <is>
-          <t>Patricio Briones</t>
+          <t>Patricio Briones Moller</t>
         </is>
       </c>
       <c r="B123" s="10" t="inlineStr">
@@ -5881,7 +5881,7 @@
     <row r="124">
       <c r="A124" s="10" t="inlineStr">
         <is>
-          <t>Patricio Pinilla</t>
+          <t>Patricio Pinilla Valencia</t>
         </is>
       </c>
       <c r="B124" s="10" t="inlineStr">
@@ -5895,16 +5895,16 @@
         </is>
       </c>
       <c r="D124" s="11" t="n">
-        <v>0.97</v>
+        <v>0.95</v>
       </c>
       <c r="E124" s="11" t="n">
-        <v>1</v>
+        <v>0.98</v>
       </c>
       <c r="F124" s="10" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G124" s="10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H124" s="12" t="n">
         <v>13674030</v>
@@ -5922,7 +5922,7 @@
     <row r="125">
       <c r="A125" s="10" t="inlineStr">
         <is>
-          <t>Paula Olmos</t>
+          <t>Paula Olmos Contreras</t>
         </is>
       </c>
       <c r="B125" s="10" t="inlineStr">
@@ -5936,10 +5936,10 @@
         </is>
       </c>
       <c r="D125" s="11" t="n">
-        <v>0.82</v>
+        <v>0.83</v>
       </c>
       <c r="E125" s="11" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.95</v>
       </c>
       <c r="F125" s="10" t="n">
         <v>13</v>
@@ -5963,7 +5963,7 @@
     <row r="126">
       <c r="A126" s="10" t="inlineStr">
         <is>
-          <t>Paulina Muñoz</t>
+          <t>Paulina Muñoz Minte</t>
         </is>
       </c>
       <c r="B126" s="10" t="inlineStr">
@@ -6004,7 +6004,7 @@
     <row r="127">
       <c r="A127" s="10" t="inlineStr">
         <is>
-          <t>Paz Charpentier</t>
+          <t>Paz Charpentier Rajcevich</t>
         </is>
       </c>
       <c r="B127" s="10" t="inlineStr">
@@ -6045,7 +6045,7 @@
     <row r="128">
       <c r="A128" s="10" t="inlineStr">
         <is>
-          <t>Pier Karlezi</t>
+          <t>Pier Karlezi Hazleby</t>
         </is>
       </c>
       <c r="B128" s="10" t="inlineStr">
@@ -6059,7 +6059,7 @@
         </is>
       </c>
       <c r="D128" s="11" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.95</v>
       </c>
       <c r="E128" s="11" t="n">
         <v>0.98</v>
@@ -6086,7 +6086,7 @@
     <row r="129">
       <c r="A129" s="10" t="inlineStr">
         <is>
-          <t>Priscilla Castillo</t>
+          <t>Priscilla Castillo Gerli</t>
         </is>
       </c>
       <c r="B129" s="10" t="inlineStr">
@@ -6127,7 +6127,7 @@
     <row r="130">
       <c r="A130" s="10" t="inlineStr">
         <is>
-          <t>Raúl Leiva</t>
+          <t>Raúl Leiva Carvajal</t>
         </is>
       </c>
       <c r="B130" s="10" t="inlineStr">
@@ -6141,16 +6141,16 @@
         </is>
       </c>
       <c r="D130" s="11" t="n">
-        <v>0.95</v>
+        <v>0.92</v>
       </c>
       <c r="E130" s="11" t="n">
-        <v>1</v>
+        <v>0.98</v>
       </c>
       <c r="F130" s="10" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="G130" s="10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H130" s="12" t="n">
         <v>12517235</v>
@@ -6168,7 +6168,7 @@
     <row r="131">
       <c r="A131" s="10" t="inlineStr">
         <is>
-          <t>Raúl Soto</t>
+          <t>Raúl Soto Mardones</t>
         </is>
       </c>
       <c r="B131" s="10" t="inlineStr">
@@ -6182,16 +6182,16 @@
         </is>
       </c>
       <c r="D131" s="11" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.9</v>
       </c>
       <c r="E131" s="11" t="n">
-        <v>0.9399999999999999</v>
+        <v>1</v>
       </c>
       <c r="F131" s="10" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="G131" s="10" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="H131" s="12" t="n">
         <v>12704015</v>
@@ -6209,7 +6209,7 @@
     <row r="132">
       <c r="A132" s="10" t="inlineStr">
         <is>
-          <t>René Alinco</t>
+          <t>René Alinco Bustos</t>
         </is>
       </c>
       <c r="B132" s="10" t="inlineStr">
@@ -6250,7 +6250,7 @@
     <row r="133">
       <c r="A133" s="10" t="inlineStr">
         <is>
-          <t>René Manuel García</t>
+          <t>René Manuel García García</t>
         </is>
       </c>
       <c r="B133" s="10" t="inlineStr">
@@ -6264,7 +6264,7 @@
         </is>
       </c>
       <c r="D133" s="11" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.95</v>
       </c>
       <c r="E133" s="11" t="n">
         <v>1</v>
@@ -6291,7 +6291,7 @@
     <row r="134">
       <c r="A134" s="10" t="inlineStr">
         <is>
-          <t>Ricardo Neumann</t>
+          <t>Ricardo Neumann Bertín</t>
         </is>
       </c>
       <c r="B134" s="10" t="inlineStr">
@@ -6332,7 +6332,7 @@
     <row r="135">
       <c r="A135" s="10" t="inlineStr">
         <is>
-          <t>Roberto Arroyo</t>
+          <t>Roberto Arroyo Muñoz</t>
         </is>
       </c>
       <c r="B135" s="10" t="inlineStr">
@@ -6346,7 +6346,7 @@
         </is>
       </c>
       <c r="D135" s="11" t="n">
-        <v>0.86</v>
+        <v>0.87</v>
       </c>
       <c r="E135" s="11" t="n">
         <v>1</v>
@@ -6373,7 +6373,7 @@
     <row r="136">
       <c r="A136" s="10" t="inlineStr">
         <is>
-          <t>Roberto Celedón</t>
+          <t>Roberto Celedón Fernández</t>
         </is>
       </c>
       <c r="B136" s="10" t="inlineStr">
@@ -6414,7 +6414,7 @@
     <row r="137">
       <c r="A137" s="10" t="inlineStr">
         <is>
-          <t>Rodrigo Ramírez</t>
+          <t>Rodrigo Ramírez Parra</t>
         </is>
       </c>
       <c r="B137" s="10" t="inlineStr">
@@ -6455,7 +6455,7 @@
     <row r="138">
       <c r="A138" s="10" t="inlineStr">
         <is>
-          <t>Sara Concha</t>
+          <t>Sara Concha Smith</t>
         </is>
       </c>
       <c r="B138" s="10" t="inlineStr">
@@ -6496,7 +6496,7 @@
     <row r="139">
       <c r="A139" s="10" t="inlineStr">
         <is>
-          <t>Sebastián Cristoffanini</t>
+          <t>Sebastián Cristoffanini Jaraquemada</t>
         </is>
       </c>
       <c r="B139" s="10" t="inlineStr">
@@ -6537,7 +6537,7 @@
     <row r="140">
       <c r="A140" s="10" t="inlineStr">
         <is>
-          <t>Sebastián Videla</t>
+          <t>Sebastián Videla Castillo</t>
         </is>
       </c>
       <c r="B140" s="10" t="inlineStr">
@@ -6578,7 +6578,7 @@
     <row r="141">
       <c r="A141" s="10" t="inlineStr">
         <is>
-          <t>Sebastián Zamora</t>
+          <t>Sebastián Zamora Soto</t>
         </is>
       </c>
       <c r="B141" s="10" t="inlineStr">
@@ -6619,7 +6619,7 @@
     <row r="142">
       <c r="A142" s="10" t="inlineStr">
         <is>
-          <t>Sergio Bobadilla</t>
+          <t>Sergio Bobadilla Muñoz</t>
         </is>
       </c>
       <c r="B142" s="10" t="inlineStr">
@@ -6660,7 +6660,7 @@
     <row r="143">
       <c r="A143" s="10" t="inlineStr">
         <is>
-          <t>Sofía González</t>
+          <t>Sofía González Cortés</t>
         </is>
       </c>
       <c r="B143" s="10" t="inlineStr">
@@ -6674,13 +6674,13 @@
         </is>
       </c>
       <c r="D143" s="11" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.9</v>
       </c>
       <c r="E143" s="11" t="n">
         <v>0.98</v>
       </c>
       <c r="F143" s="10" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="G143" s="10" t="n">
         <v>1</v>
@@ -6701,7 +6701,7 @@
     <row r="144">
       <c r="A144" s="10" t="inlineStr">
         <is>
-          <t>Stephan Schubert</t>
+          <t>Stephan Schubert Rubio</t>
         </is>
       </c>
       <c r="B144" s="10" t="inlineStr">
@@ -6715,7 +6715,7 @@
         </is>
       </c>
       <c r="D144" s="11" t="n">
-        <v>0.87</v>
+        <v>0.88</v>
       </c>
       <c r="E144" s="11" t="n">
         <v>0.93</v>
@@ -6742,7 +6742,7 @@
     <row r="145">
       <c r="A145" s="10" t="inlineStr">
         <is>
-          <t>Stephanie Jéldrez</t>
+          <t>Stephanie Jéldrez Ortiz</t>
         </is>
       </c>
       <c r="B145" s="10" t="inlineStr">
@@ -6783,7 +6783,7 @@
     <row r="146">
       <c r="A146" s="10" t="inlineStr">
         <is>
-          <t>Tamara Ramírez</t>
+          <t>Tamara Ramírez Ramírez</t>
         </is>
       </c>
       <c r="B146" s="10" t="inlineStr">
@@ -6797,7 +6797,7 @@
         </is>
       </c>
       <c r="D146" s="11" t="n">
-        <v>0.95</v>
+        <v>0.96</v>
       </c>
       <c r="E146" s="11" t="n">
         <v>1</v>
@@ -6824,7 +6824,7 @@
     <row r="147">
       <c r="A147" s="10" t="inlineStr">
         <is>
-          <t>Tatiana Urrutia</t>
+          <t>Tatiana Urrutia Herrera</t>
         </is>
       </c>
       <c r="B147" s="10" t="inlineStr">
@@ -6838,10 +6838,10 @@
         </is>
       </c>
       <c r="D147" s="11" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.95</v>
       </c>
       <c r="E147" s="11" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.95</v>
       </c>
       <c r="F147" s="10" t="n">
         <v>4</v>
@@ -6865,7 +6865,7 @@
     <row r="148">
       <c r="A148" s="10" t="inlineStr">
         <is>
-          <t>Tomás Kast</t>
+          <t>Tomás Kast Sommerhoff</t>
         </is>
       </c>
       <c r="B148" s="10" t="inlineStr">
@@ -6906,7 +6906,7 @@
     <row r="149">
       <c r="A149" s="10" t="inlineStr">
         <is>
-          <t>Valentina Becerra</t>
+          <t>Valentina Becerra Peña</t>
         </is>
       </c>
       <c r="B149" s="10" t="inlineStr">
@@ -6947,7 +6947,7 @@
     <row r="150">
       <c r="A150" s="10" t="inlineStr">
         <is>
-          <t>Valentina Cáceres</t>
+          <t>Valentina Cáceres Monsálvez</t>
         </is>
       </c>
       <c r="B150" s="10" t="inlineStr">
@@ -6961,16 +6961,16 @@
         </is>
       </c>
       <c r="D150" s="11" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.93</v>
       </c>
       <c r="E150" s="11" t="n">
-        <v>1</v>
+        <v>0.98</v>
       </c>
       <c r="F150" s="10" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G150" s="10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H150" s="12" t="n">
         <v>15454676</v>
@@ -6988,7 +6988,7 @@
     <row r="151">
       <c r="A151" s="10" t="inlineStr">
         <is>
-          <t>Ximena Naranjo</t>
+          <t>Ximena Naranjo Pinto</t>
         </is>
       </c>
       <c r="B151" s="10" t="inlineStr">
@@ -7029,7 +7029,7 @@
     <row r="152">
       <c r="A152" s="10" t="inlineStr">
         <is>
-          <t>Ximena Ossandón</t>
+          <t>Ximena Ossandón Irarrázabal</t>
         </is>
       </c>
       <c r="B152" s="10" t="inlineStr">
@@ -7070,7 +7070,7 @@
     <row r="153">
       <c r="A153" s="10" t="inlineStr">
         <is>
-          <t>Zandra Parisi</t>
+          <t>Zandra Parisi Fernández</t>
         </is>
       </c>
       <c r="B153" s="10" t="inlineStr">
@@ -7084,7 +7084,7 @@
         </is>
       </c>
       <c r="D153" s="11" t="n">
-        <v>0.89</v>
+        <v>0.9</v>
       </c>
       <c r="E153" s="11" t="n">
         <v>1</v>
@@ -7111,7 +7111,7 @@
     <row r="154">
       <c r="A154" s="10" t="inlineStr">
         <is>
-          <t>Álvaro Carter</t>
+          <t>Álvaro Carter Fernández</t>
         </is>
       </c>
       <c r="B154" s="10" t="inlineStr">
@@ -7152,7 +7152,7 @@
     <row r="155">
       <c r="A155" s="10" t="inlineStr">
         <is>
-          <t>Álvaro Jofré</t>
+          <t>Álvaro Jofré Cáceres</t>
         </is>
       </c>
       <c r="B155" s="10" t="inlineStr">
@@ -7193,7 +7193,7 @@
     <row r="156">
       <c r="A156" s="10" t="inlineStr">
         <is>
-          <t>Álvaro Ortiz</t>
+          <t>Álvaro Ortiz Vera</t>
         </is>
       </c>
       <c r="B156" s="10" t="inlineStr">
@@ -7207,10 +7207,10 @@
         </is>
       </c>
       <c r="D156" s="11" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.95</v>
       </c>
       <c r="E156" s="11" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.95</v>
       </c>
       <c r="F156" s="10" t="n">
         <v>4</v>
@@ -7305,10 +7305,10 @@
         <v>0.97</v>
       </c>
       <c r="D2" s="12" t="n">
-        <v>2</v>
+        <v>2.3</v>
       </c>
       <c r="E2" s="12" t="n">
-        <v>0.9</v>
+        <v>1</v>
       </c>
       <c r="F2" s="12" t="n">
         <v>14893179</v>
@@ -7327,10 +7327,10 @@
         <v>28</v>
       </c>
       <c r="C3" s="11" t="n">
-        <v>0.965</v>
+        <v>0.961</v>
       </c>
       <c r="D3" s="12" t="n">
-        <v>2.3</v>
+        <v>2.8</v>
       </c>
       <c r="E3" s="12" t="n">
         <v>1</v>
@@ -7345,51 +7345,51 @@
     <row r="4">
       <c r="A4" s="10" t="inlineStr">
         <is>
-          <t>UDI</t>
+          <t>PS/PL/PR</t>
         </is>
       </c>
       <c r="B4" s="10" t="n">
         <v>13</v>
       </c>
       <c r="C4" s="11" t="n">
-        <v>0.9640000000000001</v>
+        <v>0.96</v>
       </c>
       <c r="D4" s="12" t="n">
-        <v>2.5</v>
+        <v>3</v>
       </c>
       <c r="E4" s="12" t="n">
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="F4" s="12" t="n">
-        <v>13348033</v>
+        <v>15233287</v>
       </c>
       <c r="G4" s="12" t="n">
-        <v>173524429</v>
+        <v>198032731</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="10" t="inlineStr">
         <is>
-          <t>PS/PL/PR</t>
+          <t>UDI</t>
         </is>
       </c>
       <c r="B5" s="10" t="n">
         <v>13</v>
       </c>
       <c r="C5" s="11" t="n">
-        <v>0.9590000000000001</v>
+        <v>0.958</v>
       </c>
       <c r="D5" s="12" t="n">
-        <v>2.7</v>
+        <v>3.3</v>
       </c>
       <c r="E5" s="12" t="n">
         <v>0.8</v>
       </c>
       <c r="F5" s="12" t="n">
-        <v>15233287</v>
+        <v>13348033</v>
       </c>
       <c r="G5" s="12" t="n">
-        <v>198032731</v>
+        <v>173524429</v>
       </c>
     </row>
     <row r="6">
@@ -7402,13 +7402,13 @@
         <v>4</v>
       </c>
       <c r="C6" s="11" t="n">
-        <v>0.958</v>
+        <v>0.9520000000000001</v>
       </c>
       <c r="D6" s="12" t="n">
-        <v>2.8</v>
+        <v>3.8</v>
       </c>
       <c r="E6" s="12" t="n">
-        <v>1.8</v>
+        <v>0.8</v>
       </c>
       <c r="F6" s="12" t="n">
         <v>14929578</v>
@@ -7427,13 +7427,13 @@
         <v>13</v>
       </c>
       <c r="C7" s="11" t="n">
-        <v>0.948</v>
+        <v>0.9440000000000001</v>
       </c>
       <c r="D7" s="12" t="n">
-        <v>3.5</v>
+        <v>4.2</v>
       </c>
       <c r="E7" s="12" t="n">
-        <v>1.2</v>
+        <v>1.7</v>
       </c>
       <c r="F7" s="12" t="n">
         <v>14989029</v>
@@ -7445,76 +7445,76 @@
     <row r="8">
       <c r="A8" s="10" t="inlineStr">
         <is>
-          <t>PNL</t>
+          <t>Independientes</t>
         </is>
       </c>
       <c r="B8" s="10" t="n">
-        <v>8</v>
+        <v>29</v>
       </c>
       <c r="C8" s="11" t="n">
-        <v>0.945</v>
+        <v>0.9429999999999999</v>
       </c>
       <c r="D8" s="12" t="n">
-        <v>3.8</v>
+        <v>4.4</v>
       </c>
       <c r="E8" s="12" t="n">
-        <v>1.9</v>
+        <v>1.2</v>
       </c>
       <c r="F8" s="12" t="n">
-        <v>14164351</v>
+        <v>14636885</v>
       </c>
       <c r="G8" s="12" t="n">
-        <v>113314808</v>
+        <v>424469665</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="10" t="inlineStr">
         <is>
-          <t>Independientes</t>
+          <t>PNL</t>
         </is>
       </c>
       <c r="B9" s="10" t="n">
-        <v>29</v>
+        <v>8</v>
       </c>
       <c r="C9" s="11" t="n">
-        <v>0.9420000000000001</v>
+        <v>0.9379999999999999</v>
       </c>
       <c r="D9" s="12" t="n">
-        <v>4.1</v>
+        <v>4.8</v>
       </c>
       <c r="E9" s="12" t="n">
-        <v>1</v>
+        <v>2.2</v>
       </c>
       <c r="F9" s="12" t="n">
-        <v>14636885</v>
+        <v>14164351</v>
       </c>
       <c r="G9" s="12" t="n">
-        <v>424469665</v>
+        <v>113314808</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="10" t="inlineStr">
         <is>
-          <t>Comunistas</t>
+          <t>PDG</t>
         </is>
       </c>
       <c r="B10" s="10" t="n">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="C10" s="11" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.9309999999999999</v>
       </c>
       <c r="D10" s="12" t="n">
-        <v>4.2</v>
+        <v>5.3</v>
       </c>
       <c r="E10" s="12" t="n">
-        <v>1.2</v>
+        <v>0.9</v>
       </c>
       <c r="F10" s="12" t="n">
-        <v>15236021</v>
+        <v>14875781</v>
       </c>
       <c r="G10" s="12" t="n">
-        <v>137124189</v>
+        <v>208260934</v>
       </c>
     </row>
     <row r="11">
@@ -7545,26 +7545,26 @@
     <row r="12">
       <c r="A12" s="10" t="inlineStr">
         <is>
-          <t>PDG</t>
+          <t>Comunistas</t>
         </is>
       </c>
       <c r="B12" s="10" t="n">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="C12" s="11" t="n">
         <v>0.929</v>
       </c>
       <c r="D12" s="12" t="n">
-        <v>5</v>
+        <v>5.6</v>
       </c>
       <c r="E12" s="12" t="n">
-        <v>1.1</v>
+        <v>1.3</v>
       </c>
       <c r="F12" s="12" t="n">
-        <v>14875781</v>
+        <v>15236021</v>
       </c>
       <c r="G12" s="12" t="n">
-        <v>208260934</v>
+        <v>137124189</v>
       </c>
     </row>
     <row r="13">
@@ -7577,10 +7577,10 @@
         <v>16</v>
       </c>
       <c r="C13" s="11" t="n">
-        <v>0.7959999999999999</v>
+        <v>0.794</v>
       </c>
       <c r="D13" s="12" t="n">
-        <v>14.6</v>
+        <v>16.2</v>
       </c>
       <c r="E13" s="12" t="n">
         <v>1.4</v>
@@ -7603,7 +7603,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C34"/>
+  <dimension ref="A1:C35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -7637,7 +7637,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>618</v>
+        <v>632</v>
       </c>
     </row>
     <row r="5">
@@ -7647,7 +7647,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>179</v>
+        <v>200</v>
       </c>
     </row>
     <row r="6">
@@ -7657,7 +7657,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>149</v>
+        <v>163</v>
       </c>
     </row>
     <row r="7">
@@ -7667,7 +7667,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>30</v>
+        <v>33</v>
       </c>
     </row>
     <row r="9">
@@ -7689,7 +7689,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>777</v>
+        <v>814</v>
       </c>
     </row>
     <row r="11">
@@ -7699,7 +7699,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>199</v>
+        <v>214</v>
       </c>
     </row>
     <row r="13">
@@ -7791,181 +7791,191 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-10</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
         <is>
           <t>Los proyectos con más votaciones del año</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr"/>
-    </row>
-    <row r="24">
-      <c r="A24" s="9" t="inlineStr">
+      <c r="B24" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="9" t="inlineStr">
         <is>
           <t>Boletín</t>
         </is>
       </c>
-      <c r="B24" s="9" t="inlineStr">
+      <c r="B25" s="9" t="inlineStr">
         <is>
           <t>Nombre del proyecto</t>
         </is>
       </c>
-      <c r="C24" s="9" t="inlineStr">
+      <c r="C25" s="9" t="inlineStr">
         <is>
           <t>N° de votaciones</t>
         </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>18216-05</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>Para la reconstrucción nacional y el desarrollo económico y social</t>
-        </is>
-      </c>
-      <c r="C25" t="n">
-        <v>120</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>18036-05</t>
+          <t>18216-05</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Otorga reajuste general de remuneraciones a las y los trabajadores del sector público, concede aguinaldos que señala, concede otros beneficios que indica y modifica diversos cuerpos legales</t>
+          <t>Para la reconstrucción nacional y el desarrollo económico y social</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>74</v>
+        <v>120</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>16781-04</t>
+          <t>18036-05</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Modifica la ley N° 20.370, General de Educación, para crear la figura del coordinador de buena convivencia escolar</t>
+          <t>Otorga reajuste general de remuneraciones a las y los trabajadores del sector público, concede aguinaldos que señala, concede otros beneficios que indica y modifica diversos cuerpos legales</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>38</v>
+        <v>74</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>18156-04</t>
+          <t>16781-04</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Establece medidas de seguridad, orden y respeto para la comunidad educativa</t>
+          <t>Modifica la ley N° 20.370, General de Educación, para crear la figura del coordinador de buena convivencia escolar</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>31</v>
+        <v>38</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>18384-08</t>
+          <t>18156-04</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Ley de protección tarifaria eléctrica</t>
+          <t>Establece medidas de seguridad, orden y respeto para la comunidad educativa</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>16</v>
+        <v>31</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>17640-06</t>
+          <t>18384-08</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Modifica diversos cuerpos legales, para promover la gobernabilidad y la representatividad del sistema político</t>
+          <t>Ley de protección tarifaria eléctrica</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>12</v>
+        <v>16</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>16743-04</t>
+          <t>17640-06</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Modifica diversos cuerpos legales, con el objeto de facilitar la creación de nuevos establecimientos educacionales</t>
+          <t>Modifica diversos cuerpos legales, para promover la gobernabilidad y la representatividad del sistema político</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>16335-14</t>
+          <t>16743-04</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Regula la prevención y mitigación de incendios forestales, y otras materias que indica</t>
+          <t>Modifica diversos cuerpos legales, con el objeto de facilitar la creación de nuevos establecimientos educacionales</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>16857-07</t>
+          <t>16335-14</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Modifica el Código Penal para autorizar el uso de agentes encubiertos en Internet para la persecución de delitos sexuales contra niños, niñas y adolescentes</t>
+          <t>Regula la prevención y mitigación de incendios forestales, y otras materias que indica</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
+          <t>16857-07</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Modifica el Código Penal para autorizar el uso de agentes encubiertos en Internet para la persecución de delitos sexuales contra niños, niñas y adolescentes</t>
+        </is>
+      </c>
+      <c r="C34" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
           <t>18137-05</t>
         </is>
       </c>
-      <c r="B34" t="inlineStr">
+      <c r="B35" t="inlineStr">
         <is>
           <t>Adopta medidas transitorias para contener el precio del kerosene doméstico en el contexto de la emergencia energética internacional, y otras medidas que indica</t>
         </is>
       </c>
-      <c r="C34" t="n">
+      <c r="C35" t="n">
         <v>9</v>
       </c>
     </row>
@@ -9284,7 +9294,7 @@
         <v>0.97</v>
       </c>
       <c r="H2" s="11" t="n">
-        <v>0.97</v>
+        <v>0.92</v>
       </c>
       <c r="I2" s="11" t="n">
         <v>0.97</v>
@@ -9474,7 +9484,7 @@
         <v>1</v>
       </c>
       <c r="H7" s="11" t="n">
-        <v>0.89</v>
+        <v>0.86</v>
       </c>
       <c r="I7" s="11" t="n">
         <v>1</v>
@@ -9588,14 +9598,14 @@
         <v>1</v>
       </c>
       <c r="H10" s="11" t="n">
-        <v>0.82</v>
+        <v>0.75</v>
       </c>
       <c r="I10" s="11" t="n">
-        <v>1</v>
+        <v>0.95</v>
       </c>
       <c r="J10" s="10" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No (licencias/permisos)</t>
         </is>
       </c>
     </row>
@@ -9626,7 +9636,7 @@
         <v>1</v>
       </c>
       <c r="H11" s="11" t="n">
-        <v>1</v>
+        <v>0.97</v>
       </c>
       <c r="I11" s="11" t="n">
         <v>1</v>
@@ -9664,10 +9674,10 @@
         <v>1</v>
       </c>
       <c r="H12" s="11" t="n">
-        <v>0.98</v>
+        <v>0.96</v>
       </c>
       <c r="I12" s="11" t="n">
-        <v>0.98</v>
+        <v>0.97</v>
       </c>
       <c r="J12" s="10" t="inlineStr">
         <is>
@@ -9702,7 +9712,7 @@
         <v>1</v>
       </c>
       <c r="H13" s="11" t="n">
-        <v>0.9</v>
+        <v>0.91</v>
       </c>
       <c r="I13" s="11" t="n">
         <v>1</v>
@@ -9740,7 +9750,7 @@
         <v>1</v>
       </c>
       <c r="H14" s="11" t="n">
-        <v>0.93</v>
+        <v>0.85</v>
       </c>
       <c r="I14" s="11" t="n">
         <v>1</v>
@@ -9930,10 +9940,10 @@
         <v>0.955</v>
       </c>
       <c r="H19" s="11" t="n">
-        <v>0.95</v>
+        <v>0.96</v>
       </c>
       <c r="I19" s="11" t="n">
-        <v>0.95</v>
+        <v>0.96</v>
       </c>
       <c r="J19" s="10" t="inlineStr">
         <is>
@@ -10044,7 +10054,7 @@
         <v>0.973</v>
       </c>
       <c r="H22" s="11" t="n">
-        <v>0.86</v>
+        <v>0.87</v>
       </c>
       <c r="I22" s="11" t="n">
         <v>0.97</v>
@@ -10082,14 +10092,14 @@
         <v>0.9409999999999999</v>
       </c>
       <c r="H23" s="11" t="n">
-        <v>0.95</v>
+        <v>0.96</v>
       </c>
       <c r="I23" s="11" t="n">
-        <v>0.95</v>
+        <v>0.96</v>
       </c>
       <c r="J23" s="10" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No (licencias/permisos)</t>
         </is>
       </c>
     </row>
@@ -10158,7 +10168,7 @@
         <v>1</v>
       </c>
       <c r="H25" s="11" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.95</v>
       </c>
       <c r="I25" s="11" t="n">
         <v>1</v>
@@ -10196,7 +10206,7 @@
         <v>0.985</v>
       </c>
       <c r="H26" s="11" t="n">
-        <v>0.45</v>
+        <v>0.41</v>
       </c>
       <c r="I26" s="11" t="n">
         <v>0.98</v>
@@ -10272,7 +10282,7 @@
         <v>1</v>
       </c>
       <c r="H28" s="11" t="n">
-        <v>0.95</v>
+        <v>0.96</v>
       </c>
       <c r="I28" s="11" t="n">
         <v>1</v>
@@ -10310,14 +10320,14 @@
         <v>0.955</v>
       </c>
       <c r="H29" s="11" t="n">
-        <v>0.91</v>
+        <v>0.92</v>
       </c>
       <c r="I29" s="11" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.95</v>
       </c>
       <c r="J29" s="10" t="inlineStr">
         <is>
-          <t>No (licencias/permisos)</t>
+          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -10424,7 +10434,7 @@
         <v>1</v>
       </c>
       <c r="H32" s="11" t="n">
-        <v>0.95</v>
+        <v>0.96</v>
       </c>
       <c r="I32" s="11" t="n">
         <v>1</v>
@@ -10500,10 +10510,10 @@
         <v>0.9129999999999999</v>
       </c>
       <c r="H34" s="11" t="n">
-        <v>0.91</v>
+        <v>0.92</v>
       </c>
       <c r="I34" s="11" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.95</v>
       </c>
       <c r="J34" s="10" t="inlineStr">
         <is>
@@ -10538,14 +10548,14 @@
         <v>0.97</v>
       </c>
       <c r="H35" s="11" t="n">
-        <v>0.89</v>
+        <v>0.88</v>
       </c>
       <c r="I35" s="11" t="n">
-        <v>0.95</v>
+        <v>0.96</v>
       </c>
       <c r="J35" s="10" t="inlineStr">
         <is>
-          <t>No (licencias/permisos)</t>
+          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -10576,7 +10586,7 @@
         <v>1</v>
       </c>
       <c r="H36" s="11" t="n">
-        <v>0.95</v>
+        <v>0.91</v>
       </c>
       <c r="I36" s="11" t="n">
         <v>1</v>
@@ -10614,14 +10624,14 @@
         <v>0.97</v>
       </c>
       <c r="H37" s="11" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.95</v>
       </c>
       <c r="I37" s="11" t="n">
-        <v>0.95</v>
+        <v>0.96</v>
       </c>
       <c r="J37" s="10" t="inlineStr">
         <is>
-          <t>No (licencias/permisos)</t>
+          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -10769,11 +10779,11 @@
         <v>0.9</v>
       </c>
       <c r="I41" s="11" t="n">
-        <v>0.98</v>
+        <v>1</v>
       </c>
       <c r="J41" s="10" t="inlineStr">
         <is>
-          <t>No (licencias/permisos)</t>
+          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -10804,10 +10814,10 @@
         <v>0.955</v>
       </c>
       <c r="H42" s="11" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.95</v>
       </c>
       <c r="I42" s="11" t="n">
-        <v>0.95</v>
+        <v>0.96</v>
       </c>
       <c r="J42" s="10" t="inlineStr">
         <is>
@@ -10880,10 +10890,10 @@
         <v>0.887</v>
       </c>
       <c r="H44" s="11" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.95</v>
       </c>
       <c r="I44" s="11" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.95</v>
       </c>
       <c r="J44" s="10" t="inlineStr">
         <is>
@@ -11184,14 +11194,14 @@
         <v>0.955</v>
       </c>
       <c r="H52" s="11" t="n">
-        <v>0.91</v>
+        <v>0.88</v>
       </c>
       <c r="I52" s="11" t="n">
-        <v>0.95</v>
+        <v>0.93</v>
       </c>
       <c r="J52" s="10" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No (licencias/permisos)</t>
         </is>
       </c>
     </row>
@@ -11222,10 +11232,10 @@
         <v>0.955</v>
       </c>
       <c r="H53" s="11" t="n">
-        <v>0.95</v>
+        <v>0.96</v>
       </c>
       <c r="I53" s="11" t="n">
-        <v>0.95</v>
+        <v>0.96</v>
       </c>
       <c r="J53" s="10" t="inlineStr">
         <is>
@@ -11260,7 +11270,7 @@
         <v>0.973</v>
       </c>
       <c r="H54" s="11" t="n">
-        <v>0.91</v>
+        <v>0.92</v>
       </c>
       <c r="I54" s="11" t="n">
         <v>1</v>
@@ -11374,7 +11384,7 @@
         <v>1</v>
       </c>
       <c r="H57" s="11" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.95</v>
       </c>
       <c r="I57" s="11" t="n">
         <v>1</v>
@@ -11450,7 +11460,7 @@
         <v>1</v>
       </c>
       <c r="H59" s="11" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.9</v>
       </c>
       <c r="I59" s="11" t="n">
         <v>1</v>
@@ -11488,7 +11498,7 @@
         <v>1</v>
       </c>
       <c r="H60" s="11" t="n">
-        <v>0.95</v>
+        <v>0.97</v>
       </c>
       <c r="I60" s="11" t="n">
         <v>1</v>
@@ -11602,14 +11612,14 @@
         <v>0.955</v>
       </c>
       <c r="H63" s="11" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.95</v>
       </c>
       <c r="I63" s="11" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.95</v>
       </c>
       <c r="J63" s="10" t="inlineStr">
         <is>
-          <t>No (licencias/permisos)</t>
+          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -11716,10 +11726,10 @@
         <v>0.892</v>
       </c>
       <c r="H66" s="11" t="n">
-        <v>0.83</v>
+        <v>0.78</v>
       </c>
       <c r="I66" s="11" t="n">
-        <v>0.93</v>
+        <v>0.92</v>
       </c>
       <c r="J66" s="10" t="inlineStr">
         <is>
@@ -11754,7 +11764,7 @@
         <v>0.985</v>
       </c>
       <c r="H67" s="11" t="n">
-        <v>0.91</v>
+        <v>0.92</v>
       </c>
       <c r="I67" s="11" t="n">
         <v>0.98</v>
@@ -11792,14 +11802,14 @@
         <v>0.955</v>
       </c>
       <c r="H68" s="11" t="n">
-        <v>0.89</v>
+        <v>0.9</v>
       </c>
       <c r="I68" s="11" t="n">
-        <v>0.9</v>
+        <v>0.96</v>
       </c>
       <c r="J68" s="10" t="inlineStr">
         <is>
-          <t>No (licencias/permisos)</t>
+          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -11944,10 +11954,10 @@
         <v>0.9279999999999999</v>
       </c>
       <c r="H72" s="11" t="n">
-        <v>0.89</v>
+        <v>0.88</v>
       </c>
       <c r="I72" s="11" t="n">
-        <v>0.93</v>
+        <v>0.92</v>
       </c>
       <c r="J72" s="10" t="inlineStr">
         <is>
@@ -11982,7 +11992,7 @@
         <v>0.986</v>
       </c>
       <c r="H73" s="11" t="n">
-        <v>0.91</v>
+        <v>0.92</v>
       </c>
       <c r="I73" s="11" t="n">
         <v>0.98</v>
@@ -12020,7 +12030,7 @@
         <v>1</v>
       </c>
       <c r="H74" s="11" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.95</v>
       </c>
       <c r="I74" s="11" t="n">
         <v>1</v>
@@ -12096,7 +12106,7 @@
         <v>1</v>
       </c>
       <c r="H76" s="11" t="n">
-        <v>1</v>
+        <v>0.95</v>
       </c>
       <c r="I76" s="11" t="n">
         <v>1</v>
@@ -12175,7 +12185,7 @@
         <v>0.93</v>
       </c>
       <c r="I78" s="11" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.95</v>
       </c>
       <c r="J78" s="10" t="inlineStr">
         <is>
@@ -12286,7 +12296,7 @@
         <v>0.97</v>
       </c>
       <c r="H81" s="11" t="n">
-        <v>0.89</v>
+        <v>0.9</v>
       </c>
       <c r="I81" s="11" t="n">
         <v>0.97</v>
@@ -12400,7 +12410,7 @@
         <v>1</v>
       </c>
       <c r="H84" s="11" t="n">
-        <v>0.08</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="I84" s="11" t="n">
         <v>1</v>
@@ -12479,7 +12489,7 @@
         <v>0.93</v>
       </c>
       <c r="I86" s="11" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.95</v>
       </c>
       <c r="J86" s="10" t="inlineStr">
         <is>
@@ -12514,14 +12524,14 @@
         <v>0.986</v>
       </c>
       <c r="H87" s="11" t="n">
-        <v>0.93</v>
+        <v>0.91</v>
       </c>
       <c r="I87" s="11" t="n">
-        <v>0.98</v>
+        <v>0.97</v>
       </c>
       <c r="J87" s="10" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No (licencias/permisos)</t>
         </is>
       </c>
     </row>
@@ -12552,7 +12562,7 @@
         <v>1</v>
       </c>
       <c r="H88" s="11" t="n">
-        <v>0.78</v>
+        <v>0.75</v>
       </c>
       <c r="I88" s="11" t="n">
         <v>1</v>
@@ -12742,7 +12752,7 @@
         <v>1</v>
       </c>
       <c r="H93" s="11" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.95</v>
       </c>
       <c r="I93" s="11" t="n">
         <v>1</v>
@@ -12780,7 +12790,7 @@
         <v>1</v>
       </c>
       <c r="H94" s="11" t="n">
-        <v>0.95</v>
+        <v>0.96</v>
       </c>
       <c r="I94" s="11" t="n">
         <v>1</v>
@@ -12821,11 +12831,11 @@
         <v>0.91</v>
       </c>
       <c r="I95" s="11" t="n">
-        <v>1</v>
+        <v>0.98</v>
       </c>
       <c r="J95" s="10" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No (licencias/permisos)</t>
         </is>
       </c>
     </row>
@@ -12894,10 +12904,10 @@
         <v>0.97</v>
       </c>
       <c r="H97" s="11" t="n">
-        <v>0.97</v>
+        <v>0.96</v>
       </c>
       <c r="I97" s="11" t="n">
-        <v>0.97</v>
+        <v>0.96</v>
       </c>
       <c r="J97" s="10" t="inlineStr">
         <is>
@@ -12932,10 +12942,10 @@
         <v>0.9399999999999999</v>
       </c>
       <c r="H98" s="11" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.95</v>
       </c>
       <c r="I98" s="11" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.95</v>
       </c>
       <c r="J98" s="10" t="inlineStr">
         <is>
@@ -13008,14 +13018,14 @@
         <v>1</v>
       </c>
       <c r="H100" s="11" t="n">
-        <v>0.49</v>
+        <v>0.5</v>
       </c>
       <c r="I100" s="11" t="n">
-        <v>0.9399999999999999</v>
+        <v>1</v>
       </c>
       <c r="J100" s="10" t="inlineStr">
         <is>
-          <t>No (licencias/permisos)</t>
+          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -13198,14 +13208,14 @@
         <v>1</v>
       </c>
       <c r="H105" s="11" t="n">
+        <v>0.97</v>
+      </c>
+      <c r="I105" s="11" t="n">
         <v>0.98</v>
       </c>
-      <c r="I105" s="11" t="n">
-        <v>1</v>
-      </c>
       <c r="J105" s="10" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No (licencias/permisos)</t>
         </is>
       </c>
     </row>
@@ -13312,7 +13322,7 @@
         <v>1</v>
       </c>
       <c r="H108" s="11" t="n">
-        <v>0.9</v>
+        <v>0.91</v>
       </c>
       <c r="I108" s="11" t="n">
         <v>1</v>
@@ -13426,7 +13436,7 @@
         <v>1</v>
       </c>
       <c r="H111" s="11" t="n">
-        <v>0.91</v>
+        <v>0.92</v>
       </c>
       <c r="I111" s="11" t="n">
         <v>1</v>
@@ -13464,7 +13474,7 @@
         <v>0.925</v>
       </c>
       <c r="H112" s="11" t="n">
-        <v>0.89</v>
+        <v>0.9</v>
       </c>
       <c r="I112" s="11" t="n">
         <v>0.93</v>
@@ -13502,7 +13512,7 @@
         <v>1</v>
       </c>
       <c r="H113" s="11" t="n">
-        <v>0.83</v>
+        <v>0.86</v>
       </c>
       <c r="I113" s="11" t="n">
         <v>0.98</v>
@@ -13540,10 +13550,10 @@
         <v>0.985</v>
       </c>
       <c r="H114" s="11" t="n">
-        <v>0.72</v>
+        <v>0.71</v>
       </c>
       <c r="I114" s="11" t="n">
-        <v>0.93</v>
+        <v>0.9</v>
       </c>
       <c r="J114" s="10" t="inlineStr">
         <is>
@@ -13654,14 +13664,14 @@
         <v>0.8809999999999999</v>
       </c>
       <c r="H117" s="11" t="n">
-        <v>0.89</v>
+        <v>0.9</v>
       </c>
       <c r="I117" s="11" t="n">
-        <v>0.89</v>
+        <v>0.9</v>
       </c>
       <c r="J117" s="10" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No (licencias/permisos)</t>
         </is>
       </c>
     </row>
@@ -13730,10 +13740,10 @@
         <v>0.9440000000000001</v>
       </c>
       <c r="H119" s="11" t="n">
-        <v>0.75</v>
+        <v>0.76</v>
       </c>
       <c r="I119" s="11" t="n">
-        <v>0.93</v>
+        <v>0.92</v>
       </c>
       <c r="J119" s="10" t="inlineStr">
         <is>
@@ -13768,10 +13778,10 @@
         <v>0.915</v>
       </c>
       <c r="H120" s="11" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.95</v>
       </c>
       <c r="I120" s="11" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.95</v>
       </c>
       <c r="J120" s="10" t="inlineStr">
         <is>
@@ -13920,14 +13930,14 @@
         <v>1</v>
       </c>
       <c r="H124" s="11" t="n">
-        <v>0.97</v>
+        <v>0.95</v>
       </c>
       <c r="I124" s="11" t="n">
-        <v>1</v>
+        <v>0.98</v>
       </c>
       <c r="J124" s="10" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No (licencias/permisos)</t>
         </is>
       </c>
     </row>
@@ -13958,10 +13968,10 @@
         <v>0.9399999999999999</v>
       </c>
       <c r="H125" s="11" t="n">
-        <v>0.82</v>
+        <v>0.83</v>
       </c>
       <c r="I125" s="11" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.95</v>
       </c>
       <c r="J125" s="10" t="inlineStr">
         <is>
@@ -14072,7 +14082,7 @@
         <v>0.985</v>
       </c>
       <c r="H128" s="11" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.95</v>
       </c>
       <c r="I128" s="11" t="n">
         <v>0.98</v>
@@ -14148,14 +14158,14 @@
         <v>1</v>
       </c>
       <c r="H130" s="11" t="n">
-        <v>0.95</v>
+        <v>0.92</v>
       </c>
       <c r="I130" s="11" t="n">
-        <v>1</v>
+        <v>0.98</v>
       </c>
       <c r="J130" s="10" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No (licencias/permisos)</t>
         </is>
       </c>
     </row>
@@ -14186,14 +14196,14 @@
         <v>1</v>
       </c>
       <c r="H131" s="11" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.9</v>
       </c>
       <c r="I131" s="11" t="n">
-        <v>0.9399999999999999</v>
+        <v>1</v>
       </c>
       <c r="J131" s="10" t="inlineStr">
         <is>
-          <t>No (licencias/permisos)</t>
+          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -14262,7 +14272,7 @@
         <v>1</v>
       </c>
       <c r="H133" s="11" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.95</v>
       </c>
       <c r="I133" s="11" t="n">
         <v>1</v>
@@ -14338,7 +14348,7 @@
         <v>1</v>
       </c>
       <c r="H135" s="11" t="n">
-        <v>0.86</v>
+        <v>0.87</v>
       </c>
       <c r="I135" s="11" t="n">
         <v>1</v>
@@ -14642,7 +14652,7 @@
         <v>1</v>
       </c>
       <c r="H143" s="11" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.9</v>
       </c>
       <c r="I143" s="11" t="n">
         <v>0.98</v>
@@ -14680,7 +14690,7 @@
         <v>0.985</v>
       </c>
       <c r="H144" s="11" t="n">
-        <v>0.87</v>
+        <v>0.88</v>
       </c>
       <c r="I144" s="11" t="n">
         <v>0.93</v>
@@ -14756,7 +14766,7 @@
         <v>1</v>
       </c>
       <c r="H146" s="11" t="n">
-        <v>0.95</v>
+        <v>0.96</v>
       </c>
       <c r="I146" s="11" t="n">
         <v>1</v>
@@ -14794,10 +14804,10 @@
         <v>0.9399999999999999</v>
       </c>
       <c r="H147" s="11" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.95</v>
       </c>
       <c r="I147" s="11" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.95</v>
       </c>
       <c r="J147" s="10" t="inlineStr">
         <is>
@@ -14908,14 +14918,14 @@
         <v>1</v>
       </c>
       <c r="H150" s="11" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.93</v>
       </c>
       <c r="I150" s="11" t="n">
-        <v>1</v>
+        <v>0.98</v>
       </c>
       <c r="J150" s="10" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No (licencias/permisos)</t>
         </is>
       </c>
     </row>
@@ -15022,7 +15032,7 @@
         <v>1</v>
       </c>
       <c r="H153" s="11" t="n">
-        <v>0.89</v>
+        <v>0.9</v>
       </c>
       <c r="I153" s="11" t="n">
         <v>1</v>
@@ -15136,10 +15146,10 @@
         <v>1</v>
       </c>
       <c r="H156" s="11" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.95</v>
       </c>
       <c r="I156" s="11" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.95</v>
       </c>
       <c r="J156" s="10" t="inlineStr">
         <is>
@@ -15150,7 +15160,7 @@
     <row r="158">
       <c r="A158" s="15" t="inlineStr">
         <is>
-          <t>Conclusión: 130 de 155 diputad@s coinciden con el dato oficial en menos de 1 punto porcentual.</t>
+          <t>Conclusión: 128 de 155 diputad@s coinciden con el dato oficial en menos de 1 punto porcentual.</t>
         </is>
       </c>
     </row>

</xml_diff>